<commit_message>
W02 Saturday paper and key rebuilt: 55 items in six parts at 120 minutes
Built with scripts/build_saturday_paper.py W02 --docx on the source above: the
markdown paper and key, both Word files, and the item-analysis workbook with
its recalc manifest, which xlsx_recalc.py passes. The blueprint reads 8 easy,
34 medium and 13 hard.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P7zaoR4dQ5pzBFnsX549JQ
</commit_message>
<xml_diff>
--- a/content/W02/SAT/answer-key/C2_W02_SAT_item_analysis_TRAINER.xlsx
+++ b/content/W02/SAT/answer-key/C2_W02_SAT_item_analysis_TRAINER.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BD39"/>
+  <dimension ref="A1:BG39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -677,6 +677,15 @@
       <c r="BA2" t="n">
         <v>6</v>
       </c>
+      <c r="BB2" t="n">
+        <v>6</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>6</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -941,6 +950,21 @@
       </c>
       <c r="BA3" t="inlineStr">
         <is>
+          <t>[D]</t>
+        </is>
+      </c>
+      <c r="BB3" t="inlineStr">
+        <is>
+          <t>[S]</t>
+        </is>
+      </c>
+      <c r="BC3" t="inlineStr">
+        <is>
+          <t>[S]</t>
+        </is>
+      </c>
+      <c r="BD3" t="inlineStr">
+        <is>
           <t>[S]</t>
         </is>
       </c>
@@ -1213,15 +1237,30 @@
       </c>
       <c r="BB4" s="4" t="inlineStr">
         <is>
+          <t>Q53</t>
+        </is>
+      </c>
+      <c r="BC4" s="4" t="inlineStr">
+        <is>
+          <t>Q54</t>
+        </is>
+      </c>
+      <c r="BD4" s="4" t="inlineStr">
+        <is>
+          <t>Q55</t>
+        </is>
+      </c>
+      <c r="BE4" s="4" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="BC4" s="4" t="inlineStr">
+      <c r="BF4" s="4" t="inlineStr">
         <is>
           <t>Answered</t>
         </is>
       </c>
-      <c r="BD4" s="4" t="inlineStr">
+      <c r="BG4" s="4" t="inlineStr">
         <is>
           <t>Band</t>
         </is>
@@ -1283,16 +1322,19 @@
       <c r="AY5" s="5" t="n"/>
       <c r="AZ5" s="5" t="n"/>
       <c r="BA5" s="5" t="n"/>
-      <c r="BB5">
-        <f>IF(COUNT(B5:BA5)=0,"",SUM(B5:BA5))</f>
-        <v/>
-      </c>
-      <c r="BC5">
-        <f>COUNT(B5:BA5)</f>
-        <v/>
-      </c>
-      <c r="BD5">
-        <f>IF(OR(BB5="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB5,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB5,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB5" s="5" t="n"/>
+      <c r="BC5" s="5" t="n"/>
+      <c r="BD5" s="5" t="n"/>
+      <c r="BE5">
+        <f>IF(COUNT(B5:BD5)=0,"",SUM(B5:BD5))</f>
+        <v/>
+      </c>
+      <c r="BF5">
+        <f>COUNT(B5:BD5)</f>
+        <v/>
+      </c>
+      <c r="BG5">
+        <f>IF(OR(BE5="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE5,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE5,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1352,16 +1394,19 @@
       <c r="AY6" s="5" t="n"/>
       <c r="AZ6" s="5" t="n"/>
       <c r="BA6" s="5" t="n"/>
-      <c r="BB6">
-        <f>IF(COUNT(B6:BA6)=0,"",SUM(B6:BA6))</f>
-        <v/>
-      </c>
-      <c r="BC6">
-        <f>COUNT(B6:BA6)</f>
-        <v/>
-      </c>
-      <c r="BD6">
-        <f>IF(OR(BB6="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB6,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB6,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB6" s="5" t="n"/>
+      <c r="BC6" s="5" t="n"/>
+      <c r="BD6" s="5" t="n"/>
+      <c r="BE6">
+        <f>IF(COUNT(B6:BD6)=0,"",SUM(B6:BD6))</f>
+        <v/>
+      </c>
+      <c r="BF6">
+        <f>COUNT(B6:BD6)</f>
+        <v/>
+      </c>
+      <c r="BG6">
+        <f>IF(OR(BE6="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE6,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE6,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1421,16 +1466,19 @@
       <c r="AY7" s="5" t="n"/>
       <c r="AZ7" s="5" t="n"/>
       <c r="BA7" s="5" t="n"/>
-      <c r="BB7">
-        <f>IF(COUNT(B7:BA7)=0,"",SUM(B7:BA7))</f>
-        <v/>
-      </c>
-      <c r="BC7">
-        <f>COUNT(B7:BA7)</f>
-        <v/>
-      </c>
-      <c r="BD7">
-        <f>IF(OR(BB7="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB7,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB7,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB7" s="5" t="n"/>
+      <c r="BC7" s="5" t="n"/>
+      <c r="BD7" s="5" t="n"/>
+      <c r="BE7">
+        <f>IF(COUNT(B7:BD7)=0,"",SUM(B7:BD7))</f>
+        <v/>
+      </c>
+      <c r="BF7">
+        <f>COUNT(B7:BD7)</f>
+        <v/>
+      </c>
+      <c r="BG7">
+        <f>IF(OR(BE7="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE7,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE7,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1490,16 +1538,19 @@
       <c r="AY8" s="5" t="n"/>
       <c r="AZ8" s="5" t="n"/>
       <c r="BA8" s="5" t="n"/>
-      <c r="BB8">
-        <f>IF(COUNT(B8:BA8)=0,"",SUM(B8:BA8))</f>
-        <v/>
-      </c>
-      <c r="BC8">
-        <f>COUNT(B8:BA8)</f>
-        <v/>
-      </c>
-      <c r="BD8">
-        <f>IF(OR(BB8="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB8,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB8,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB8" s="5" t="n"/>
+      <c r="BC8" s="5" t="n"/>
+      <c r="BD8" s="5" t="n"/>
+      <c r="BE8">
+        <f>IF(COUNT(B8:BD8)=0,"",SUM(B8:BD8))</f>
+        <v/>
+      </c>
+      <c r="BF8">
+        <f>COUNT(B8:BD8)</f>
+        <v/>
+      </c>
+      <c r="BG8">
+        <f>IF(OR(BE8="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE8,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE8,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1559,16 +1610,19 @@
       <c r="AY9" s="5" t="n"/>
       <c r="AZ9" s="5" t="n"/>
       <c r="BA9" s="5" t="n"/>
-      <c r="BB9">
-        <f>IF(COUNT(B9:BA9)=0,"",SUM(B9:BA9))</f>
-        <v/>
-      </c>
-      <c r="BC9">
-        <f>COUNT(B9:BA9)</f>
-        <v/>
-      </c>
-      <c r="BD9">
-        <f>IF(OR(BB9="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB9,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB9,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB9" s="5" t="n"/>
+      <c r="BC9" s="5" t="n"/>
+      <c r="BD9" s="5" t="n"/>
+      <c r="BE9">
+        <f>IF(COUNT(B9:BD9)=0,"",SUM(B9:BD9))</f>
+        <v/>
+      </c>
+      <c r="BF9">
+        <f>COUNT(B9:BD9)</f>
+        <v/>
+      </c>
+      <c r="BG9">
+        <f>IF(OR(BE9="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE9,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE9,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1628,16 +1682,19 @@
       <c r="AY10" s="5" t="n"/>
       <c r="AZ10" s="5" t="n"/>
       <c r="BA10" s="5" t="n"/>
-      <c r="BB10">
-        <f>IF(COUNT(B10:BA10)=0,"",SUM(B10:BA10))</f>
-        <v/>
-      </c>
-      <c r="BC10">
-        <f>COUNT(B10:BA10)</f>
-        <v/>
-      </c>
-      <c r="BD10">
-        <f>IF(OR(BB10="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB10,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB10,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB10" s="5" t="n"/>
+      <c r="BC10" s="5" t="n"/>
+      <c r="BD10" s="5" t="n"/>
+      <c r="BE10">
+        <f>IF(COUNT(B10:BD10)=0,"",SUM(B10:BD10))</f>
+        <v/>
+      </c>
+      <c r="BF10">
+        <f>COUNT(B10:BD10)</f>
+        <v/>
+      </c>
+      <c r="BG10">
+        <f>IF(OR(BE10="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE10,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE10,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1697,16 +1754,19 @@
       <c r="AY11" s="5" t="n"/>
       <c r="AZ11" s="5" t="n"/>
       <c r="BA11" s="5" t="n"/>
-      <c r="BB11">
-        <f>IF(COUNT(B11:BA11)=0,"",SUM(B11:BA11))</f>
-        <v/>
-      </c>
-      <c r="BC11">
-        <f>COUNT(B11:BA11)</f>
-        <v/>
-      </c>
-      <c r="BD11">
-        <f>IF(OR(BB11="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB11,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB11,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB11" s="5" t="n"/>
+      <c r="BC11" s="5" t="n"/>
+      <c r="BD11" s="5" t="n"/>
+      <c r="BE11">
+        <f>IF(COUNT(B11:BD11)=0,"",SUM(B11:BD11))</f>
+        <v/>
+      </c>
+      <c r="BF11">
+        <f>COUNT(B11:BD11)</f>
+        <v/>
+      </c>
+      <c r="BG11">
+        <f>IF(OR(BE11="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE11,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE11,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1766,16 +1826,19 @@
       <c r="AY12" s="5" t="n"/>
       <c r="AZ12" s="5" t="n"/>
       <c r="BA12" s="5" t="n"/>
-      <c r="BB12">
-        <f>IF(COUNT(B12:BA12)=0,"",SUM(B12:BA12))</f>
-        <v/>
-      </c>
-      <c r="BC12">
-        <f>COUNT(B12:BA12)</f>
-        <v/>
-      </c>
-      <c r="BD12">
-        <f>IF(OR(BB12="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB12,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB12,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB12" s="5" t="n"/>
+      <c r="BC12" s="5" t="n"/>
+      <c r="BD12" s="5" t="n"/>
+      <c r="BE12">
+        <f>IF(COUNT(B12:BD12)=0,"",SUM(B12:BD12))</f>
+        <v/>
+      </c>
+      <c r="BF12">
+        <f>COUNT(B12:BD12)</f>
+        <v/>
+      </c>
+      <c r="BG12">
+        <f>IF(OR(BE12="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE12,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE12,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1835,16 +1898,19 @@
       <c r="AY13" s="5" t="n"/>
       <c r="AZ13" s="5" t="n"/>
       <c r="BA13" s="5" t="n"/>
-      <c r="BB13">
-        <f>IF(COUNT(B13:BA13)=0,"",SUM(B13:BA13))</f>
-        <v/>
-      </c>
-      <c r="BC13">
-        <f>COUNT(B13:BA13)</f>
-        <v/>
-      </c>
-      <c r="BD13">
-        <f>IF(OR(BB13="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB13,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB13,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB13" s="5" t="n"/>
+      <c r="BC13" s="5" t="n"/>
+      <c r="BD13" s="5" t="n"/>
+      <c r="BE13">
+        <f>IF(COUNT(B13:BD13)=0,"",SUM(B13:BD13))</f>
+        <v/>
+      </c>
+      <c r="BF13">
+        <f>COUNT(B13:BD13)</f>
+        <v/>
+      </c>
+      <c r="BG13">
+        <f>IF(OR(BE13="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE13,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE13,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1904,16 +1970,19 @@
       <c r="AY14" s="5" t="n"/>
       <c r="AZ14" s="5" t="n"/>
       <c r="BA14" s="5" t="n"/>
-      <c r="BB14">
-        <f>IF(COUNT(B14:BA14)=0,"",SUM(B14:BA14))</f>
-        <v/>
-      </c>
-      <c r="BC14">
-        <f>COUNT(B14:BA14)</f>
-        <v/>
-      </c>
-      <c r="BD14">
-        <f>IF(OR(BB14="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB14,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB14,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB14" s="5" t="n"/>
+      <c r="BC14" s="5" t="n"/>
+      <c r="BD14" s="5" t="n"/>
+      <c r="BE14">
+        <f>IF(COUNT(B14:BD14)=0,"",SUM(B14:BD14))</f>
+        <v/>
+      </c>
+      <c r="BF14">
+        <f>COUNT(B14:BD14)</f>
+        <v/>
+      </c>
+      <c r="BG14">
+        <f>IF(OR(BE14="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE14,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE14,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -1973,16 +2042,19 @@
       <c r="AY15" s="5" t="n"/>
       <c r="AZ15" s="5" t="n"/>
       <c r="BA15" s="5" t="n"/>
-      <c r="BB15">
-        <f>IF(COUNT(B15:BA15)=0,"",SUM(B15:BA15))</f>
-        <v/>
-      </c>
-      <c r="BC15">
-        <f>COUNT(B15:BA15)</f>
-        <v/>
-      </c>
-      <c r="BD15">
-        <f>IF(OR(BB15="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB15,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB15,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB15" s="5" t="n"/>
+      <c r="BC15" s="5" t="n"/>
+      <c r="BD15" s="5" t="n"/>
+      <c r="BE15">
+        <f>IF(COUNT(B15:BD15)=0,"",SUM(B15:BD15))</f>
+        <v/>
+      </c>
+      <c r="BF15">
+        <f>COUNT(B15:BD15)</f>
+        <v/>
+      </c>
+      <c r="BG15">
+        <f>IF(OR(BE15="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE15,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE15,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2042,16 +2114,19 @@
       <c r="AY16" s="5" t="n"/>
       <c r="AZ16" s="5" t="n"/>
       <c r="BA16" s="5" t="n"/>
-      <c r="BB16">
-        <f>IF(COUNT(B16:BA16)=0,"",SUM(B16:BA16))</f>
-        <v/>
-      </c>
-      <c r="BC16">
-        <f>COUNT(B16:BA16)</f>
-        <v/>
-      </c>
-      <c r="BD16">
-        <f>IF(OR(BB16="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB16,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB16,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB16" s="5" t="n"/>
+      <c r="BC16" s="5" t="n"/>
+      <c r="BD16" s="5" t="n"/>
+      <c r="BE16">
+        <f>IF(COUNT(B16:BD16)=0,"",SUM(B16:BD16))</f>
+        <v/>
+      </c>
+      <c r="BF16">
+        <f>COUNT(B16:BD16)</f>
+        <v/>
+      </c>
+      <c r="BG16">
+        <f>IF(OR(BE16="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE16,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE16,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2111,16 +2186,19 @@
       <c r="AY17" s="5" t="n"/>
       <c r="AZ17" s="5" t="n"/>
       <c r="BA17" s="5" t="n"/>
-      <c r="BB17">
-        <f>IF(COUNT(B17:BA17)=0,"",SUM(B17:BA17))</f>
-        <v/>
-      </c>
-      <c r="BC17">
-        <f>COUNT(B17:BA17)</f>
-        <v/>
-      </c>
-      <c r="BD17">
-        <f>IF(OR(BB17="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB17,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB17,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB17" s="5" t="n"/>
+      <c r="BC17" s="5" t="n"/>
+      <c r="BD17" s="5" t="n"/>
+      <c r="BE17">
+        <f>IF(COUNT(B17:BD17)=0,"",SUM(B17:BD17))</f>
+        <v/>
+      </c>
+      <c r="BF17">
+        <f>COUNT(B17:BD17)</f>
+        <v/>
+      </c>
+      <c r="BG17">
+        <f>IF(OR(BE17="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE17,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE17,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2180,16 +2258,19 @@
       <c r="AY18" s="5" t="n"/>
       <c r="AZ18" s="5" t="n"/>
       <c r="BA18" s="5" t="n"/>
-      <c r="BB18">
-        <f>IF(COUNT(B18:BA18)=0,"",SUM(B18:BA18))</f>
-        <v/>
-      </c>
-      <c r="BC18">
-        <f>COUNT(B18:BA18)</f>
-        <v/>
-      </c>
-      <c r="BD18">
-        <f>IF(OR(BB18="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB18,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB18,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB18" s="5" t="n"/>
+      <c r="BC18" s="5" t="n"/>
+      <c r="BD18" s="5" t="n"/>
+      <c r="BE18">
+        <f>IF(COUNT(B18:BD18)=0,"",SUM(B18:BD18))</f>
+        <v/>
+      </c>
+      <c r="BF18">
+        <f>COUNT(B18:BD18)</f>
+        <v/>
+      </c>
+      <c r="BG18">
+        <f>IF(OR(BE18="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE18,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE18,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2249,16 +2330,19 @@
       <c r="AY19" s="5" t="n"/>
       <c r="AZ19" s="5" t="n"/>
       <c r="BA19" s="5" t="n"/>
-      <c r="BB19">
-        <f>IF(COUNT(B19:BA19)=0,"",SUM(B19:BA19))</f>
-        <v/>
-      </c>
-      <c r="BC19">
-        <f>COUNT(B19:BA19)</f>
-        <v/>
-      </c>
-      <c r="BD19">
-        <f>IF(OR(BB19="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB19,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB19,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB19" s="5" t="n"/>
+      <c r="BC19" s="5" t="n"/>
+      <c r="BD19" s="5" t="n"/>
+      <c r="BE19">
+        <f>IF(COUNT(B19:BD19)=0,"",SUM(B19:BD19))</f>
+        <v/>
+      </c>
+      <c r="BF19">
+        <f>COUNT(B19:BD19)</f>
+        <v/>
+      </c>
+      <c r="BG19">
+        <f>IF(OR(BE19="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE19,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE19,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2318,16 +2402,19 @@
       <c r="AY20" s="5" t="n"/>
       <c r="AZ20" s="5" t="n"/>
       <c r="BA20" s="5" t="n"/>
-      <c r="BB20">
-        <f>IF(COUNT(B20:BA20)=0,"",SUM(B20:BA20))</f>
-        <v/>
-      </c>
-      <c r="BC20">
-        <f>COUNT(B20:BA20)</f>
-        <v/>
-      </c>
-      <c r="BD20">
-        <f>IF(OR(BB20="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB20,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB20,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB20" s="5" t="n"/>
+      <c r="BC20" s="5" t="n"/>
+      <c r="BD20" s="5" t="n"/>
+      <c r="BE20">
+        <f>IF(COUNT(B20:BD20)=0,"",SUM(B20:BD20))</f>
+        <v/>
+      </c>
+      <c r="BF20">
+        <f>COUNT(B20:BD20)</f>
+        <v/>
+      </c>
+      <c r="BG20">
+        <f>IF(OR(BE20="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE20,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE20,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2387,16 +2474,19 @@
       <c r="AY21" s="5" t="n"/>
       <c r="AZ21" s="5" t="n"/>
       <c r="BA21" s="5" t="n"/>
-      <c r="BB21">
-        <f>IF(COUNT(B21:BA21)=0,"",SUM(B21:BA21))</f>
-        <v/>
-      </c>
-      <c r="BC21">
-        <f>COUNT(B21:BA21)</f>
-        <v/>
-      </c>
-      <c r="BD21">
-        <f>IF(OR(BB21="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB21,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB21,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB21" s="5" t="n"/>
+      <c r="BC21" s="5" t="n"/>
+      <c r="BD21" s="5" t="n"/>
+      <c r="BE21">
+        <f>IF(COUNT(B21:BD21)=0,"",SUM(B21:BD21))</f>
+        <v/>
+      </c>
+      <c r="BF21">
+        <f>COUNT(B21:BD21)</f>
+        <v/>
+      </c>
+      <c r="BG21">
+        <f>IF(OR(BE21="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE21,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE21,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2456,16 +2546,19 @@
       <c r="AY22" s="5" t="n"/>
       <c r="AZ22" s="5" t="n"/>
       <c r="BA22" s="5" t="n"/>
-      <c r="BB22">
-        <f>IF(COUNT(B22:BA22)=0,"",SUM(B22:BA22))</f>
-        <v/>
-      </c>
-      <c r="BC22">
-        <f>COUNT(B22:BA22)</f>
-        <v/>
-      </c>
-      <c r="BD22">
-        <f>IF(OR(BB22="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB22,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB22,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB22" s="5" t="n"/>
+      <c r="BC22" s="5" t="n"/>
+      <c r="BD22" s="5" t="n"/>
+      <c r="BE22">
+        <f>IF(COUNT(B22:BD22)=0,"",SUM(B22:BD22))</f>
+        <v/>
+      </c>
+      <c r="BF22">
+        <f>COUNT(B22:BD22)</f>
+        <v/>
+      </c>
+      <c r="BG22">
+        <f>IF(OR(BE22="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE22,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE22,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2525,16 +2618,19 @@
       <c r="AY23" s="5" t="n"/>
       <c r="AZ23" s="5" t="n"/>
       <c r="BA23" s="5" t="n"/>
-      <c r="BB23">
-        <f>IF(COUNT(B23:BA23)=0,"",SUM(B23:BA23))</f>
-        <v/>
-      </c>
-      <c r="BC23">
-        <f>COUNT(B23:BA23)</f>
-        <v/>
-      </c>
-      <c r="BD23">
-        <f>IF(OR(BB23="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB23,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB23,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB23" s="5" t="n"/>
+      <c r="BC23" s="5" t="n"/>
+      <c r="BD23" s="5" t="n"/>
+      <c r="BE23">
+        <f>IF(COUNT(B23:BD23)=0,"",SUM(B23:BD23))</f>
+        <v/>
+      </c>
+      <c r="BF23">
+        <f>COUNT(B23:BD23)</f>
+        <v/>
+      </c>
+      <c r="BG23">
+        <f>IF(OR(BE23="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE23,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE23,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2594,16 +2690,19 @@
       <c r="AY24" s="5" t="n"/>
       <c r="AZ24" s="5" t="n"/>
       <c r="BA24" s="5" t="n"/>
-      <c r="BB24">
-        <f>IF(COUNT(B24:BA24)=0,"",SUM(B24:BA24))</f>
-        <v/>
-      </c>
-      <c r="BC24">
-        <f>COUNT(B24:BA24)</f>
-        <v/>
-      </c>
-      <c r="BD24">
-        <f>IF(OR(BB24="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB24,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB24,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB24" s="5" t="n"/>
+      <c r="BC24" s="5" t="n"/>
+      <c r="BD24" s="5" t="n"/>
+      <c r="BE24">
+        <f>IF(COUNT(B24:BD24)=0,"",SUM(B24:BD24))</f>
+        <v/>
+      </c>
+      <c r="BF24">
+        <f>COUNT(B24:BD24)</f>
+        <v/>
+      </c>
+      <c r="BG24">
+        <f>IF(OR(BE24="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE24,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE24,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2663,16 +2762,19 @@
       <c r="AY25" s="5" t="n"/>
       <c r="AZ25" s="5" t="n"/>
       <c r="BA25" s="5" t="n"/>
-      <c r="BB25">
-        <f>IF(COUNT(B25:BA25)=0,"",SUM(B25:BA25))</f>
-        <v/>
-      </c>
-      <c r="BC25">
-        <f>COUNT(B25:BA25)</f>
-        <v/>
-      </c>
-      <c r="BD25">
-        <f>IF(OR(BB25="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB25,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB25,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB25" s="5" t="n"/>
+      <c r="BC25" s="5" t="n"/>
+      <c r="BD25" s="5" t="n"/>
+      <c r="BE25">
+        <f>IF(COUNT(B25:BD25)=0,"",SUM(B25:BD25))</f>
+        <v/>
+      </c>
+      <c r="BF25">
+        <f>COUNT(B25:BD25)</f>
+        <v/>
+      </c>
+      <c r="BG25">
+        <f>IF(OR(BE25="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE25,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE25,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2732,16 +2834,19 @@
       <c r="AY26" s="5" t="n"/>
       <c r="AZ26" s="5" t="n"/>
       <c r="BA26" s="5" t="n"/>
-      <c r="BB26">
-        <f>IF(COUNT(B26:BA26)=0,"",SUM(B26:BA26))</f>
-        <v/>
-      </c>
-      <c r="BC26">
-        <f>COUNT(B26:BA26)</f>
-        <v/>
-      </c>
-      <c r="BD26">
-        <f>IF(OR(BB26="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB26,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB26,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB26" s="5" t="n"/>
+      <c r="BC26" s="5" t="n"/>
+      <c r="BD26" s="5" t="n"/>
+      <c r="BE26">
+        <f>IF(COUNT(B26:BD26)=0,"",SUM(B26:BD26))</f>
+        <v/>
+      </c>
+      <c r="BF26">
+        <f>COUNT(B26:BD26)</f>
+        <v/>
+      </c>
+      <c r="BG26">
+        <f>IF(OR(BE26="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE26,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE26,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2801,16 +2906,19 @@
       <c r="AY27" s="5" t="n"/>
       <c r="AZ27" s="5" t="n"/>
       <c r="BA27" s="5" t="n"/>
-      <c r="BB27">
-        <f>IF(COUNT(B27:BA27)=0,"",SUM(B27:BA27))</f>
-        <v/>
-      </c>
-      <c r="BC27">
-        <f>COUNT(B27:BA27)</f>
-        <v/>
-      </c>
-      <c r="BD27">
-        <f>IF(OR(BB27="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB27,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB27,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB27" s="5" t="n"/>
+      <c r="BC27" s="5" t="n"/>
+      <c r="BD27" s="5" t="n"/>
+      <c r="BE27">
+        <f>IF(COUNT(B27:BD27)=0,"",SUM(B27:BD27))</f>
+        <v/>
+      </c>
+      <c r="BF27">
+        <f>COUNT(B27:BD27)</f>
+        <v/>
+      </c>
+      <c r="BG27">
+        <f>IF(OR(BE27="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE27,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE27,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2870,16 +2978,19 @@
       <c r="AY28" s="5" t="n"/>
       <c r="AZ28" s="5" t="n"/>
       <c r="BA28" s="5" t="n"/>
-      <c r="BB28">
-        <f>IF(COUNT(B28:BA28)=0,"",SUM(B28:BA28))</f>
-        <v/>
-      </c>
-      <c r="BC28">
-        <f>COUNT(B28:BA28)</f>
-        <v/>
-      </c>
-      <c r="BD28">
-        <f>IF(OR(BB28="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB28,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB28,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB28" s="5" t="n"/>
+      <c r="BC28" s="5" t="n"/>
+      <c r="BD28" s="5" t="n"/>
+      <c r="BE28">
+        <f>IF(COUNT(B28:BD28)=0,"",SUM(B28:BD28))</f>
+        <v/>
+      </c>
+      <c r="BF28">
+        <f>COUNT(B28:BD28)</f>
+        <v/>
+      </c>
+      <c r="BG28">
+        <f>IF(OR(BE28="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE28,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE28,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -2939,16 +3050,19 @@
       <c r="AY29" s="5" t="n"/>
       <c r="AZ29" s="5" t="n"/>
       <c r="BA29" s="5" t="n"/>
-      <c r="BB29">
-        <f>IF(COUNT(B29:BA29)=0,"",SUM(B29:BA29))</f>
-        <v/>
-      </c>
-      <c r="BC29">
-        <f>COUNT(B29:BA29)</f>
-        <v/>
-      </c>
-      <c r="BD29">
-        <f>IF(OR(BB29="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB29,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB29,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB29" s="5" t="n"/>
+      <c r="BC29" s="5" t="n"/>
+      <c r="BD29" s="5" t="n"/>
+      <c r="BE29">
+        <f>IF(COUNT(B29:BD29)=0,"",SUM(B29:BD29))</f>
+        <v/>
+      </c>
+      <c r="BF29">
+        <f>COUNT(B29:BD29)</f>
+        <v/>
+      </c>
+      <c r="BG29">
+        <f>IF(OR(BE29="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE29,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE29,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -3008,16 +3122,19 @@
       <c r="AY30" s="5" t="n"/>
       <c r="AZ30" s="5" t="n"/>
       <c r="BA30" s="5" t="n"/>
-      <c r="BB30">
-        <f>IF(COUNT(B30:BA30)=0,"",SUM(B30:BA30))</f>
-        <v/>
-      </c>
-      <c r="BC30">
-        <f>COUNT(B30:BA30)</f>
-        <v/>
-      </c>
-      <c r="BD30">
-        <f>IF(OR(BB30="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB30,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB30,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB30" s="5" t="n"/>
+      <c r="BC30" s="5" t="n"/>
+      <c r="BD30" s="5" t="n"/>
+      <c r="BE30">
+        <f>IF(COUNT(B30:BD30)=0,"",SUM(B30:BD30))</f>
+        <v/>
+      </c>
+      <c r="BF30">
+        <f>COUNT(B30:BD30)</f>
+        <v/>
+      </c>
+      <c r="BG30">
+        <f>IF(OR(BE30="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE30,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE30,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -3077,16 +3194,19 @@
       <c r="AY31" s="5" t="n"/>
       <c r="AZ31" s="5" t="n"/>
       <c r="BA31" s="5" t="n"/>
-      <c r="BB31">
-        <f>IF(COUNT(B31:BA31)=0,"",SUM(B31:BA31))</f>
-        <v/>
-      </c>
-      <c r="BC31">
-        <f>COUNT(B31:BA31)</f>
-        <v/>
-      </c>
-      <c r="BD31">
-        <f>IF(OR(BB31="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB31,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB31,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB31" s="5" t="n"/>
+      <c r="BC31" s="5" t="n"/>
+      <c r="BD31" s="5" t="n"/>
+      <c r="BE31">
+        <f>IF(COUNT(B31:BD31)=0,"",SUM(B31:BD31))</f>
+        <v/>
+      </c>
+      <c r="BF31">
+        <f>COUNT(B31:BD31)</f>
+        <v/>
+      </c>
+      <c r="BG31">
+        <f>IF(OR(BE31="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE31,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE31,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -3146,16 +3266,19 @@
       <c r="AY32" s="5" t="n"/>
       <c r="AZ32" s="5" t="n"/>
       <c r="BA32" s="5" t="n"/>
-      <c r="BB32">
-        <f>IF(COUNT(B32:BA32)=0,"",SUM(B32:BA32))</f>
-        <v/>
-      </c>
-      <c r="BC32">
-        <f>COUNT(B32:BA32)</f>
-        <v/>
-      </c>
-      <c r="BD32">
-        <f>IF(OR(BB32="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB32,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB32,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB32" s="5" t="n"/>
+      <c r="BC32" s="5" t="n"/>
+      <c r="BD32" s="5" t="n"/>
+      <c r="BE32">
+        <f>IF(COUNT(B32:BD32)=0,"",SUM(B32:BD32))</f>
+        <v/>
+      </c>
+      <c r="BF32">
+        <f>COUNT(B32:BD32)</f>
+        <v/>
+      </c>
+      <c r="BG32">
+        <f>IF(OR(BE32="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE32,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE32,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -3215,16 +3338,19 @@
       <c r="AY33" s="5" t="n"/>
       <c r="AZ33" s="5" t="n"/>
       <c r="BA33" s="5" t="n"/>
-      <c r="BB33">
-        <f>IF(COUNT(B33:BA33)=0,"",SUM(B33:BA33))</f>
-        <v/>
-      </c>
-      <c r="BC33">
-        <f>COUNT(B33:BA33)</f>
-        <v/>
-      </c>
-      <c r="BD33">
-        <f>IF(OR(BB33="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB33,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB33,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB33" s="5" t="n"/>
+      <c r="BC33" s="5" t="n"/>
+      <c r="BD33" s="5" t="n"/>
+      <c r="BE33">
+        <f>IF(COUNT(B33:BD33)=0,"",SUM(B33:BD33))</f>
+        <v/>
+      </c>
+      <c r="BF33">
+        <f>COUNT(B33:BD33)</f>
+        <v/>
+      </c>
+      <c r="BG33">
+        <f>IF(OR(BE33="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE33,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE33,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -3284,16 +3410,19 @@
       <c r="AY34" s="5" t="n"/>
       <c r="AZ34" s="5" t="n"/>
       <c r="BA34" s="5" t="n"/>
-      <c r="BB34">
-        <f>IF(COUNT(B34:BA34)=0,"",SUM(B34:BA34))</f>
-        <v/>
-      </c>
-      <c r="BC34">
-        <f>COUNT(B34:BA34)</f>
-        <v/>
-      </c>
-      <c r="BD34">
-        <f>IF(OR(BB34="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB34,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB34,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB34" s="5" t="n"/>
+      <c r="BC34" s="5" t="n"/>
+      <c r="BD34" s="5" t="n"/>
+      <c r="BE34">
+        <f>IF(COUNT(B34:BD34)=0,"",SUM(B34:BD34))</f>
+        <v/>
+      </c>
+      <c r="BF34">
+        <f>COUNT(B34:BD34)</f>
+        <v/>
+      </c>
+      <c r="BG34">
+        <f>IF(OR(BE34="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE34,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE34,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -3353,16 +3482,19 @@
       <c r="AY35" s="5" t="n"/>
       <c r="AZ35" s="5" t="n"/>
       <c r="BA35" s="5" t="n"/>
-      <c r="BB35">
-        <f>IF(COUNT(B35:BA35)=0,"",SUM(B35:BA35))</f>
-        <v/>
-      </c>
-      <c r="BC35">
-        <f>COUNT(B35:BA35)</f>
-        <v/>
-      </c>
-      <c r="BD35">
-        <f>IF(OR(BB35="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB35,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB35,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB35" s="5" t="n"/>
+      <c r="BC35" s="5" t="n"/>
+      <c r="BD35" s="5" t="n"/>
+      <c r="BE35">
+        <f>IF(COUNT(B35:BD35)=0,"",SUM(B35:BD35))</f>
+        <v/>
+      </c>
+      <c r="BF35">
+        <f>COUNT(B35:BD35)</f>
+        <v/>
+      </c>
+      <c r="BG35">
+        <f>IF(OR(BE35="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE35,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE35,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -3422,16 +3554,19 @@
       <c r="AY36" s="5" t="n"/>
       <c r="AZ36" s="5" t="n"/>
       <c r="BA36" s="5" t="n"/>
-      <c r="BB36">
-        <f>IF(COUNT(B36:BA36)=0,"",SUM(B36:BA36))</f>
-        <v/>
-      </c>
-      <c r="BC36">
-        <f>COUNT(B36:BA36)</f>
-        <v/>
-      </c>
-      <c r="BD36">
-        <f>IF(OR(BB36="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB36,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB36,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB36" s="5" t="n"/>
+      <c r="BC36" s="5" t="n"/>
+      <c r="BD36" s="5" t="n"/>
+      <c r="BE36">
+        <f>IF(COUNT(B36:BD36)=0,"",SUM(B36:BD36))</f>
+        <v/>
+      </c>
+      <c r="BF36">
+        <f>COUNT(B36:BD36)</f>
+        <v/>
+      </c>
+      <c r="BG36">
+        <f>IF(OR(BE36="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE36,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE36,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -3491,16 +3626,19 @@
       <c r="AY37" s="5" t="n"/>
       <c r="AZ37" s="5" t="n"/>
       <c r="BA37" s="5" t="n"/>
-      <c r="BB37">
-        <f>IF(COUNT(B37:BA37)=0,"",SUM(B37:BA37))</f>
-        <v/>
-      </c>
-      <c r="BC37">
-        <f>COUNT(B37:BA37)</f>
-        <v/>
-      </c>
-      <c r="BD37">
-        <f>IF(OR(BB37="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB37,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB37,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB37" s="5" t="n"/>
+      <c r="BC37" s="5" t="n"/>
+      <c r="BD37" s="5" t="n"/>
+      <c r="BE37">
+        <f>IF(COUNT(B37:BD37)=0,"",SUM(B37:BD37))</f>
+        <v/>
+      </c>
+      <c r="BF37">
+        <f>COUNT(B37:BD37)</f>
+        <v/>
+      </c>
+      <c r="BG37">
+        <f>IF(OR(BE37="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE37,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE37,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -3560,16 +3698,19 @@
       <c r="AY38" s="5" t="n"/>
       <c r="AZ38" s="5" t="n"/>
       <c r="BA38" s="5" t="n"/>
-      <c r="BB38">
-        <f>IF(COUNT(B38:BA38)=0,"",SUM(B38:BA38))</f>
-        <v/>
-      </c>
-      <c r="BC38">
-        <f>COUNT(B38:BA38)</f>
-        <v/>
-      </c>
-      <c r="BD38">
-        <f>IF(OR(BB38="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB38,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB38,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB38" s="5" t="n"/>
+      <c r="BC38" s="5" t="n"/>
+      <c r="BD38" s="5" t="n"/>
+      <c r="BE38">
+        <f>IF(COUNT(B38:BD38)=0,"",SUM(B38:BD38))</f>
+        <v/>
+      </c>
+      <c r="BF38">
+        <f>COUNT(B38:BD38)</f>
+        <v/>
+      </c>
+      <c r="BG38">
+        <f>IF(OR(BE38="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE38,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE38,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -3629,16 +3770,19 @@
       <c r="AY39" s="5" t="n"/>
       <c r="AZ39" s="5" t="n"/>
       <c r="BA39" s="5" t="n"/>
-      <c r="BB39">
-        <f>IF(COUNT(B39:BA39)=0,"",SUM(B39:BA39))</f>
-        <v/>
-      </c>
-      <c r="BC39">
-        <f>COUNT(B39:BA39)</f>
-        <v/>
-      </c>
-      <c r="BD39">
-        <f>IF(OR(BB39="",COUNT($BB$5:$BB$39)&lt;3),"",IF(RANK(BB39,$BB$5:$BB$39,0)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"top",IF(RANK(BB39,$BB$5:$BB$39,1)&lt;=ROUND(COUNT($BB$5:$BB$39)/3,0),"bottom","middle")))</f>
+      <c r="BB39" s="5" t="n"/>
+      <c r="BC39" s="5" t="n"/>
+      <c r="BD39" s="5" t="n"/>
+      <c r="BE39">
+        <f>IF(COUNT(B39:BD39)=0,"",SUM(B39:BD39))</f>
+        <v/>
+      </c>
+      <c r="BF39">
+        <f>COUNT(B39:BD39)</f>
+        <v/>
+      </c>
+      <c r="BG39">
+        <f>IF(OR(BE39="",COUNT($BE$5:$BE$39)&lt;3),"",IF(RANK(BE39,$BE$5:$BE$39,0)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"top",IF(RANK(BE39,$BE$5:$BE$39,1)&lt;=ROUND(COUNT($BE$5:$BE$39)/3,0),"bottom","middle")))</f>
         <v/>
       </c>
     </row>
@@ -3653,7 +3797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N56"/>
+  <dimension ref="A1:N59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="13" max="13"/>
@@ -3778,11 +3922,11 @@
         <v/>
       </c>
       <c r="J5" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!B$5:B$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!B$5:B$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!B$5:B$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!B$5:B$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!B$5:B$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!B$5:B$39)))</f>
         <v/>
       </c>
       <c r="K5" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!B$5:B$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!B$5:B$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!B$5:B$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!B$5:B$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!B$5:B$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!B$5:B$39)))</f>
         <v/>
       </c>
       <c r="L5" s="6">
@@ -3838,11 +3982,11 @@
         <v/>
       </c>
       <c r="J6" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!C$5:C$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!C$5:C$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!C$5:C$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!C$5:C$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!C$5:C$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!C$5:C$39)))</f>
         <v/>
       </c>
       <c r="K6" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!C$5:C$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!C$5:C$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!C$5:C$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!C$5:C$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!C$5:C$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!C$5:C$39)))</f>
         <v/>
       </c>
       <c r="L6" s="6">
@@ -3898,11 +4042,11 @@
         <v/>
       </c>
       <c r="J7" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!D$5:D$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!D$5:D$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!D$5:D$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!D$5:D$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!D$5:D$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!D$5:D$39)))</f>
         <v/>
       </c>
       <c r="K7" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!D$5:D$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!D$5:D$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!D$5:D$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!D$5:D$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!D$5:D$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!D$5:D$39)))</f>
         <v/>
       </c>
       <c r="L7" s="6">
@@ -3958,11 +4102,11 @@
         <v/>
       </c>
       <c r="J8" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!E$5:E$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!E$5:E$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!E$5:E$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!E$5:E$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!E$5:E$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!E$5:E$39)))</f>
         <v/>
       </c>
       <c r="K8" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!E$5:E$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!E$5:E$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!E$5:E$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!E$5:E$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!E$5:E$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!E$5:E$39)))</f>
         <v/>
       </c>
       <c r="L8" s="6">
@@ -4018,11 +4162,11 @@
         <v/>
       </c>
       <c r="J9" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!F$5:F$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!F$5:F$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!F$5:F$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!F$5:F$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!F$5:F$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!F$5:F$39)))</f>
         <v/>
       </c>
       <c r="K9" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!F$5:F$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!F$5:F$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!F$5:F$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!F$5:F$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!F$5:F$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!F$5:F$39)))</f>
         <v/>
       </c>
       <c r="L9" s="6">
@@ -4078,11 +4222,11 @@
         <v/>
       </c>
       <c r="J10" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!G$5:G$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!G$5:G$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!G$5:G$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!G$5:G$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!G$5:G$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!G$5:G$39)))</f>
         <v/>
       </c>
       <c r="K10" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!G$5:G$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!G$5:G$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!G$5:G$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!G$5:G$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!G$5:G$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!G$5:G$39)))</f>
         <v/>
       </c>
       <c r="L10" s="6">
@@ -4138,11 +4282,11 @@
         <v/>
       </c>
       <c r="J11" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!H$5:H$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!H$5:H$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!H$5:H$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!H$5:H$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!H$5:H$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!H$5:H$39)))</f>
         <v/>
       </c>
       <c r="K11" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!H$5:H$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!H$5:H$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!H$5:H$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!H$5:H$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!H$5:H$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!H$5:H$39)))</f>
         <v/>
       </c>
       <c r="L11" s="6">
@@ -4198,11 +4342,11 @@
         <v/>
       </c>
       <c r="J12" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!I$5:I$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!I$5:I$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!I$5:I$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!I$5:I$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!I$5:I$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!I$5:I$39)))</f>
         <v/>
       </c>
       <c r="K12" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!I$5:I$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!I$5:I$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!I$5:I$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!I$5:I$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!I$5:I$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!I$5:I$39)))</f>
         <v/>
       </c>
       <c r="L12" s="6">
@@ -4258,11 +4402,11 @@
         <v/>
       </c>
       <c r="J13" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!J$5:J$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!J$5:J$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!J$5:J$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!J$5:J$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!J$5:J$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!J$5:J$39)))</f>
         <v/>
       </c>
       <c r="K13" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!J$5:J$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!J$5:J$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!J$5:J$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!J$5:J$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!J$5:J$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!J$5:J$39)))</f>
         <v/>
       </c>
       <c r="L13" s="6">
@@ -4318,11 +4462,11 @@
         <v/>
       </c>
       <c r="J14" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!K$5:K$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!K$5:K$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!K$5:K$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!K$5:K$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!K$5:K$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!K$5:K$39)))</f>
         <v/>
       </c>
       <c r="K14" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!K$5:K$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!K$5:K$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!K$5:K$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!K$5:K$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!K$5:K$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!K$5:K$39)))</f>
         <v/>
       </c>
       <c r="L14" s="6">
@@ -4378,11 +4522,11 @@
         <v/>
       </c>
       <c r="J15" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!L$5:L$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!L$5:L$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!L$5:L$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!L$5:L$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!L$5:L$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!L$5:L$39)))</f>
         <v/>
       </c>
       <c r="K15" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!L$5:L$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!L$5:L$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!L$5:L$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!L$5:L$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!L$5:L$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!L$5:L$39)))</f>
         <v/>
       </c>
       <c r="L15" s="6">
@@ -4438,11 +4582,11 @@
         <v/>
       </c>
       <c r="J16" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!M$5:M$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!M$5:M$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!M$5:M$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!M$5:M$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!M$5:M$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!M$5:M$39)))</f>
         <v/>
       </c>
       <c r="K16" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!M$5:M$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!M$5:M$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!M$5:M$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!M$5:M$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!M$5:M$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!M$5:M$39)))</f>
         <v/>
       </c>
       <c r="L16" s="6">
@@ -4498,11 +4642,11 @@
         <v/>
       </c>
       <c r="J17" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!N$5:N$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!N$5:N$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!N$5:N$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!N$5:N$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!N$5:N$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!N$5:N$39)))</f>
         <v/>
       </c>
       <c r="K17" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!N$5:N$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!N$5:N$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!N$5:N$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!N$5:N$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!N$5:N$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!N$5:N$39)))</f>
         <v/>
       </c>
       <c r="L17" s="6">
@@ -4558,11 +4702,11 @@
         <v/>
       </c>
       <c r="J18" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!O$5:O$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!O$5:O$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!O$5:O$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!O$5:O$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!O$5:O$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!O$5:O$39)))</f>
         <v/>
       </c>
       <c r="K18" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!O$5:O$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!O$5:O$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!O$5:O$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!O$5:O$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!O$5:O$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!O$5:O$39)))</f>
         <v/>
       </c>
       <c r="L18" s="6">
@@ -4618,11 +4762,11 @@
         <v/>
       </c>
       <c r="J19" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!P$5:P$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!P$5:P$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!P$5:P$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!P$5:P$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!P$5:P$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!P$5:P$39)))</f>
         <v/>
       </c>
       <c r="K19" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!P$5:P$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!P$5:P$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!P$5:P$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!P$5:P$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!P$5:P$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!P$5:P$39)))</f>
         <v/>
       </c>
       <c r="L19" s="6">
@@ -4678,11 +4822,11 @@
         <v/>
       </c>
       <c r="J20" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!Q$5:Q$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!Q$5:Q$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!Q$5:Q$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!Q$5:Q$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!Q$5:Q$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!Q$5:Q$39)))</f>
         <v/>
       </c>
       <c r="K20" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!Q$5:Q$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!Q$5:Q$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!Q$5:Q$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!Q$5:Q$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!Q$5:Q$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!Q$5:Q$39)))</f>
         <v/>
       </c>
       <c r="L20" s="6">
@@ -4738,11 +4882,11 @@
         <v/>
       </c>
       <c r="J21" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!R$5:R$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!R$5:R$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!R$5:R$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!R$5:R$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!R$5:R$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!R$5:R$39)))</f>
         <v/>
       </c>
       <c r="K21" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!R$5:R$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!R$5:R$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!R$5:R$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!R$5:R$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!R$5:R$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!R$5:R$39)))</f>
         <v/>
       </c>
       <c r="L21" s="6">
@@ -4798,11 +4942,11 @@
         <v/>
       </c>
       <c r="J22" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!S$5:S$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!S$5:S$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!S$5:S$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!S$5:S$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!S$5:S$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!S$5:S$39)))</f>
         <v/>
       </c>
       <c r="K22" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!S$5:S$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!S$5:S$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!S$5:S$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!S$5:S$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!S$5:S$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!S$5:S$39)))</f>
         <v/>
       </c>
       <c r="L22" s="6">
@@ -4858,11 +5002,11 @@
         <v/>
       </c>
       <c r="J23" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!T$5:T$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!T$5:T$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!T$5:T$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!T$5:T$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!T$5:T$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!T$5:T$39)))</f>
         <v/>
       </c>
       <c r="K23" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!T$5:T$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!T$5:T$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!T$5:T$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!T$5:T$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!T$5:T$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!T$5:T$39)))</f>
         <v/>
       </c>
       <c r="L23" s="6">
@@ -4918,11 +5062,11 @@
         <v/>
       </c>
       <c r="J24" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!U$5:U$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!U$5:U$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!U$5:U$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!U$5:U$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!U$5:U$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!U$5:U$39)))</f>
         <v/>
       </c>
       <c r="K24" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!U$5:U$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!U$5:U$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!U$5:U$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!U$5:U$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!U$5:U$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!U$5:U$39)))</f>
         <v/>
       </c>
       <c r="L24" s="6">
@@ -4978,11 +5122,11 @@
         <v/>
       </c>
       <c r="J25" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!V$5:V$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!V$5:V$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!V$5:V$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!V$5:V$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!V$5:V$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!V$5:V$39)))</f>
         <v/>
       </c>
       <c r="K25" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!V$5:V$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!V$5:V$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!V$5:V$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!V$5:V$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!V$5:V$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!V$5:V$39)))</f>
         <v/>
       </c>
       <c r="L25" s="6">
@@ -5038,11 +5182,11 @@
         <v/>
       </c>
       <c r="J26" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!W$5:W$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!W$5:W$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!W$5:W$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!W$5:W$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!W$5:W$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!W$5:W$39)))</f>
         <v/>
       </c>
       <c r="K26" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!W$5:W$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!W$5:W$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!W$5:W$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!W$5:W$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!W$5:W$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!W$5:W$39)))</f>
         <v/>
       </c>
       <c r="L26" s="6">
@@ -5098,11 +5242,11 @@
         <v/>
       </c>
       <c r="J27" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!X$5:X$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!X$5:X$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!X$5:X$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!X$5:X$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!X$5:X$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!X$5:X$39)))</f>
         <v/>
       </c>
       <c r="K27" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!X$5:X$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!X$5:X$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!X$5:X$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!X$5:X$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!X$5:X$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!X$5:X$39)))</f>
         <v/>
       </c>
       <c r="L27" s="6">
@@ -5158,11 +5302,11 @@
         <v/>
       </c>
       <c r="J28" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!Y$5:Y$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!Y$5:Y$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!Y$5:Y$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!Y$5:Y$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!Y$5:Y$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!Y$5:Y$39)))</f>
         <v/>
       </c>
       <c r="K28" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!Y$5:Y$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!Y$5:Y$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!Y$5:Y$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!Y$5:Y$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!Y$5:Y$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!Y$5:Y$39)))</f>
         <v/>
       </c>
       <c r="L28" s="6">
@@ -5218,11 +5362,11 @@
         <v/>
       </c>
       <c r="J29" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!Z$5:Z$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!Z$5:Z$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!Z$5:Z$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!Z$5:Z$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!Z$5:Z$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!Z$5:Z$39)))</f>
         <v/>
       </c>
       <c r="K29" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!Z$5:Z$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!Z$5:Z$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!Z$5:Z$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!Z$5:Z$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!Z$5:Z$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!Z$5:Z$39)))</f>
         <v/>
       </c>
       <c r="L29" s="6">
@@ -5278,11 +5422,11 @@
         <v/>
       </c>
       <c r="J30" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AA$5:AA$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AA$5:AA$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AA$5:AA$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AA$5:AA$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AA$5:AA$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AA$5:AA$39)))</f>
         <v/>
       </c>
       <c r="K30" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AA$5:AA$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AA$5:AA$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AA$5:AA$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AA$5:AA$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AA$5:AA$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AA$5:AA$39)))</f>
         <v/>
       </c>
       <c r="L30" s="6">
@@ -5338,11 +5482,11 @@
         <v/>
       </c>
       <c r="J31" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AB$5:AB$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AB$5:AB$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AB$5:AB$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AB$5:AB$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AB$5:AB$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AB$5:AB$39)))</f>
         <v/>
       </c>
       <c r="K31" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AB$5:AB$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AB$5:AB$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AB$5:AB$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AB$5:AB$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AB$5:AB$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AB$5:AB$39)))</f>
         <v/>
       </c>
       <c r="L31" s="6">
@@ -5398,11 +5542,11 @@
         <v/>
       </c>
       <c r="J32" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AC$5:AC$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AC$5:AC$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AC$5:AC$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AC$5:AC$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AC$5:AC$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AC$5:AC$39)))</f>
         <v/>
       </c>
       <c r="K32" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AC$5:AC$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AC$5:AC$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AC$5:AC$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AC$5:AC$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AC$5:AC$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AC$5:AC$39)))</f>
         <v/>
       </c>
       <c r="L32" s="6">
@@ -5458,11 +5602,11 @@
         <v/>
       </c>
       <c r="J33" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AD$5:AD$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AD$5:AD$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AD$5:AD$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AD$5:AD$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AD$5:AD$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AD$5:AD$39)))</f>
         <v/>
       </c>
       <c r="K33" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AD$5:AD$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AD$5:AD$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AD$5:AD$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AD$5:AD$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AD$5:AD$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AD$5:AD$39)))</f>
         <v/>
       </c>
       <c r="L33" s="6">
@@ -5518,11 +5662,11 @@
         <v/>
       </c>
       <c r="J34" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AE$5:AE$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AE$5:AE$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AE$5:AE$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AE$5:AE$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AE$5:AE$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AE$5:AE$39)))</f>
         <v/>
       </c>
       <c r="K34" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AE$5:AE$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AE$5:AE$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AE$5:AE$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AE$5:AE$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AE$5:AE$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AE$5:AE$39)))</f>
         <v/>
       </c>
       <c r="L34" s="6">
@@ -5578,11 +5722,11 @@
         <v/>
       </c>
       <c r="J35" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AF$5:AF$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AF$5:AF$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AF$5:AF$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AF$5:AF$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AF$5:AF$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AF$5:AF$39)))</f>
         <v/>
       </c>
       <c r="K35" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AF$5:AF$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AF$5:AF$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AF$5:AF$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AF$5:AF$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AF$5:AF$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AF$5:AF$39)))</f>
         <v/>
       </c>
       <c r="L35" s="6">
@@ -5638,11 +5782,11 @@
         <v/>
       </c>
       <c r="J36" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AG$5:AG$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AG$5:AG$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AG$5:AG$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AG$5:AG$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AG$5:AG$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AG$5:AG$39)))</f>
         <v/>
       </c>
       <c r="K36" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AG$5:AG$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AG$5:AG$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AG$5:AG$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AG$5:AG$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AG$5:AG$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AG$5:AG$39)))</f>
         <v/>
       </c>
       <c r="L36" s="6">
@@ -5698,11 +5842,11 @@
         <v/>
       </c>
       <c r="J37" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AH$5:AH$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AH$5:AH$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AH$5:AH$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AH$5:AH$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AH$5:AH$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AH$5:AH$39)))</f>
         <v/>
       </c>
       <c r="K37" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AH$5:AH$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AH$5:AH$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AH$5:AH$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AH$5:AH$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AH$5:AH$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AH$5:AH$39)))</f>
         <v/>
       </c>
       <c r="L37" s="6">
@@ -5758,11 +5902,11 @@
         <v/>
       </c>
       <c r="J38" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AI$5:AI$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AI$5:AI$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AI$5:AI$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AI$5:AI$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AI$5:AI$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AI$5:AI$39)))</f>
         <v/>
       </c>
       <c r="K38" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AI$5:AI$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AI$5:AI$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AI$5:AI$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AI$5:AI$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AI$5:AI$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AI$5:AI$39)))</f>
         <v/>
       </c>
       <c r="L38" s="6">
@@ -5818,11 +5962,11 @@
         <v/>
       </c>
       <c r="J39" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AJ$5:AJ$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AJ$5:AJ$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AJ$5:AJ$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AJ$5:AJ$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AJ$5:AJ$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AJ$5:AJ$39)))</f>
         <v/>
       </c>
       <c r="K39" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AJ$5:AJ$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AJ$5:AJ$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AJ$5:AJ$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AJ$5:AJ$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AJ$5:AJ$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AJ$5:AJ$39)))</f>
         <v/>
       </c>
       <c r="L39" s="6">
@@ -5878,11 +6022,11 @@
         <v/>
       </c>
       <c r="J40" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AK$5:AK$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AK$5:AK$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AK$5:AK$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AK$5:AK$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AK$5:AK$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AK$5:AK$39)))</f>
         <v/>
       </c>
       <c r="K40" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AK$5:AK$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AK$5:AK$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AK$5:AK$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AK$5:AK$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AK$5:AK$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AK$5:AK$39)))</f>
         <v/>
       </c>
       <c r="L40" s="6">
@@ -5938,11 +6082,11 @@
         <v/>
       </c>
       <c r="J41" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AL$5:AL$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AL$5:AL$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AL$5:AL$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AL$5:AL$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AL$5:AL$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AL$5:AL$39)))</f>
         <v/>
       </c>
       <c r="K41" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AL$5:AL$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AL$5:AL$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AL$5:AL$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AL$5:AL$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AL$5:AL$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AL$5:AL$39)))</f>
         <v/>
       </c>
       <c r="L41" s="6">
@@ -5998,11 +6142,11 @@
         <v/>
       </c>
       <c r="J42" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AM$5:AM$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AM$5:AM$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AM$5:AM$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AM$5:AM$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AM$5:AM$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AM$5:AM$39)))</f>
         <v/>
       </c>
       <c r="K42" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AM$5:AM$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AM$5:AM$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AM$5:AM$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AM$5:AM$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AM$5:AM$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AM$5:AM$39)))</f>
         <v/>
       </c>
       <c r="L42" s="6">
@@ -6058,11 +6202,11 @@
         <v/>
       </c>
       <c r="J43" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AN$5:AN$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AN$5:AN$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AN$5:AN$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AN$5:AN$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AN$5:AN$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AN$5:AN$39)))</f>
         <v/>
       </c>
       <c r="K43" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AN$5:AN$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AN$5:AN$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AN$5:AN$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AN$5:AN$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AN$5:AN$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AN$5:AN$39)))</f>
         <v/>
       </c>
       <c r="L43" s="6">
@@ -6118,11 +6262,11 @@
         <v/>
       </c>
       <c r="J44" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AO$5:AO$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AO$5:AO$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AO$5:AO$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AO$5:AO$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AO$5:AO$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AO$5:AO$39)))</f>
         <v/>
       </c>
       <c r="K44" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AO$5:AO$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AO$5:AO$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AO$5:AO$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AO$5:AO$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AO$5:AO$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AO$5:AO$39)))</f>
         <v/>
       </c>
       <c r="L44" s="6">
@@ -6178,11 +6322,11 @@
         <v/>
       </c>
       <c r="J45" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AP$5:AP$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AP$5:AP$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AP$5:AP$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AP$5:AP$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AP$5:AP$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AP$5:AP$39)))</f>
         <v/>
       </c>
       <c r="K45" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AP$5:AP$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AP$5:AP$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AP$5:AP$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AP$5:AP$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AP$5:AP$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AP$5:AP$39)))</f>
         <v/>
       </c>
       <c r="L45" s="6">
@@ -6238,11 +6382,11 @@
         <v/>
       </c>
       <c r="J46" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AQ$5:AQ$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AQ$5:AQ$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AQ$5:AQ$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AQ$5:AQ$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AQ$5:AQ$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AQ$5:AQ$39)))</f>
         <v/>
       </c>
       <c r="K46" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AQ$5:AQ$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AQ$5:AQ$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AQ$5:AQ$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AQ$5:AQ$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AQ$5:AQ$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AQ$5:AQ$39)))</f>
         <v/>
       </c>
       <c r="L46" s="6">
@@ -6298,11 +6442,11 @@
         <v/>
       </c>
       <c r="J47" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AR$5:AR$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AR$5:AR$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AR$5:AR$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AR$5:AR$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AR$5:AR$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AR$5:AR$39)))</f>
         <v/>
       </c>
       <c r="K47" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AR$5:AR$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AR$5:AR$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AR$5:AR$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AR$5:AR$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AR$5:AR$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AR$5:AR$39)))</f>
         <v/>
       </c>
       <c r="L47" s="6">
@@ -6358,11 +6502,11 @@
         <v/>
       </c>
       <c r="J48" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AS$5:AS$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AS$5:AS$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AS$5:AS$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AS$5:AS$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AS$5:AS$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AS$5:AS$39)))</f>
         <v/>
       </c>
       <c r="K48" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AS$5:AS$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AS$5:AS$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AS$5:AS$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AS$5:AS$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AS$5:AS$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AS$5:AS$39)))</f>
         <v/>
       </c>
       <c r="L48" s="6">
@@ -6418,11 +6562,11 @@
         <v/>
       </c>
       <c r="J49" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AT$5:AT$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AT$5:AT$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AT$5:AT$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AT$5:AT$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AT$5:AT$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AT$5:AT$39)))</f>
         <v/>
       </c>
       <c r="K49" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AT$5:AT$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AT$5:AT$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AT$5:AT$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AT$5:AT$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AT$5:AT$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AT$5:AT$39)))</f>
         <v/>
       </c>
       <c r="L49" s="6">
@@ -6478,11 +6622,11 @@
         <v/>
       </c>
       <c r="J50" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AU$5:AU$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AU$5:AU$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AU$5:AU$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AU$5:AU$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AU$5:AU$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AU$5:AU$39)))</f>
         <v/>
       </c>
       <c r="K50" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AU$5:AU$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AU$5:AU$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AU$5:AU$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AU$5:AU$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AU$5:AU$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AU$5:AU$39)))</f>
         <v/>
       </c>
       <c r="L50" s="6">
@@ -6538,11 +6682,11 @@
         <v/>
       </c>
       <c r="J51" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AV$5:AV$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AV$5:AV$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AV$5:AV$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AV$5:AV$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AV$5:AV$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AV$5:AV$39)))</f>
         <v/>
       </c>
       <c r="K51" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AV$5:AV$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AV$5:AV$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AV$5:AV$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AV$5:AV$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AV$5:AV$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AV$5:AV$39)))</f>
         <v/>
       </c>
       <c r="L51" s="6">
@@ -6598,11 +6742,11 @@
         <v/>
       </c>
       <c r="J52" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AW$5:AW$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AW$5:AW$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AW$5:AW$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AW$5:AW$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AW$5:AW$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AW$5:AW$39)))</f>
         <v/>
       </c>
       <c r="K52" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AW$5:AW$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AW$5:AW$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AW$5:AW$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AW$5:AW$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AW$5:AW$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AW$5:AW$39)))</f>
         <v/>
       </c>
       <c r="L52" s="6">
@@ -6658,11 +6802,11 @@
         <v/>
       </c>
       <c r="J53" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AX$5:AX$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AX$5:AX$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AX$5:AX$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AX$5:AX$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AX$5:AX$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AX$5:AX$39)))</f>
         <v/>
       </c>
       <c r="K53" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AX$5:AX$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AX$5:AX$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AX$5:AX$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AX$5:AX$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AX$5:AX$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AX$5:AX$39)))</f>
         <v/>
       </c>
       <c r="L53" s="6">
@@ -6718,11 +6862,11 @@
         <v/>
       </c>
       <c r="J54" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AY$5:AY$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AY$5:AY$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AY$5:AY$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AY$5:AY$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AY$5:AY$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AY$5:AY$39)))</f>
         <v/>
       </c>
       <c r="K54" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AY$5:AY$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AY$5:AY$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AY$5:AY$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AY$5:AY$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AY$5:AY$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AY$5:AY$39)))</f>
         <v/>
       </c>
       <c r="L54" s="6">
@@ -6778,11 +6922,11 @@
         <v/>
       </c>
       <c r="J55" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AZ$5:AZ$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!AZ$5:AZ$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!AZ$5:AZ$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AZ$5:AZ$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!AZ$5:AZ$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!AZ$5:AZ$39)))</f>
         <v/>
       </c>
       <c r="K55" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AZ$5:AZ$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!AZ$5:AZ$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!AZ$5:AZ$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AZ$5:AZ$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!AZ$5:AZ$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!AZ$5:AZ$39)))</f>
         <v/>
       </c>
       <c r="L55" s="6">
@@ -6812,17 +6956,17 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>[S]</t>
+          <t>[D]</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>c</t>
         </is>
       </c>
       <c r="G56">
@@ -6838,11 +6982,11 @@
         <v/>
       </c>
       <c r="J56" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!BA$5:BA$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="top")*(Marks!BA$5:BA$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="top")*ISNUMBER(Marks!BA$5:BA$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!BA$5:BA$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!BA$5:BA$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!BA$5:BA$39)))</f>
         <v/>
       </c>
       <c r="K56" s="6">
-        <f>IF(SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!BA$5:BA$39))=0,"",SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*(Marks!BA$5:BA$39=1))/SUMPRODUCT((Marks!$BD$5:$BD$39="bottom")*ISNUMBER(Marks!BA$5:BA$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!BA$5:BA$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!BA$5:BA$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!BA$5:BA$39)))</f>
         <v/>
       </c>
       <c r="L56" s="6">
@@ -6855,6 +6999,186 @@
       </c>
       <c r="N56">
         <f>IF(H56=0,"",I56+ROW()/1000000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>53</v>
+      </c>
+      <c r="B57" t="n">
+        <v>6</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Scenario set</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>[S]</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
+      <c r="G57">
+        <f>COUNTIF(Marks!BB$5:BB$39,1)</f>
+        <v/>
+      </c>
+      <c r="H57">
+        <f>COUNT(Marks!BB$5:BB$39)</f>
+        <v/>
+      </c>
+      <c r="I57" s="6">
+        <f>IF(H57=0,"",G57/H57)</f>
+        <v/>
+      </c>
+      <c r="J57" s="6">
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!BB$5:BB$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!BB$5:BB$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!BB$5:BB$39)))</f>
+        <v/>
+      </c>
+      <c r="K57" s="6">
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!BB$5:BB$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!BB$5:BB$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!BB$5:BB$39)))</f>
+        <v/>
+      </c>
+      <c r="L57" s="6">
+        <f>IF(OR(J57="",K57=""),"",J57-K57)</f>
+        <v/>
+      </c>
+      <c r="M57">
+        <f>IF(H57=0,"",IF(I57&lt;0.2,"Check the item: fewer than one in five got it right",IF(AND(L57&lt;&gt;"",N(L57)&lt;0),"Check the item: the bottom third beat the top third","")))</f>
+        <v/>
+      </c>
+      <c r="N57">
+        <f>IF(H57=0,"",I57+ROW()/1000000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>54</v>
+      </c>
+      <c r="B58" t="n">
+        <v>6</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>One correct option</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>[S]</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>d</t>
+        </is>
+      </c>
+      <c r="G58">
+        <f>COUNTIF(Marks!BC$5:BC$39,1)</f>
+        <v/>
+      </c>
+      <c r="H58">
+        <f>COUNT(Marks!BC$5:BC$39)</f>
+        <v/>
+      </c>
+      <c r="I58" s="6">
+        <f>IF(H58=0,"",G58/H58)</f>
+        <v/>
+      </c>
+      <c r="J58" s="6">
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!BC$5:BC$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!BC$5:BC$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!BC$5:BC$39)))</f>
+        <v/>
+      </c>
+      <c r="K58" s="6">
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!BC$5:BC$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!BC$5:BC$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!BC$5:BC$39)))</f>
+        <v/>
+      </c>
+      <c r="L58" s="6">
+        <f>IF(OR(J58="",K58=""),"",J58-K58)</f>
+        <v/>
+      </c>
+      <c r="M58">
+        <f>IF(H58=0,"",IF(I58&lt;0.2,"Check the item: fewer than one in five got it right",IF(AND(L58&lt;&gt;"",N(L58)&lt;0),"Check the item: the bottom third beat the top third","")))</f>
+        <v/>
+      </c>
+      <c r="N58">
+        <f>IF(H58=0,"",I58+ROW()/1000000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>55</v>
+      </c>
+      <c r="B59" t="n">
+        <v>6</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>One correct option</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>[S]</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="G59">
+        <f>COUNTIF(Marks!BD$5:BD$39,1)</f>
+        <v/>
+      </c>
+      <c r="H59">
+        <f>COUNT(Marks!BD$5:BD$39)</f>
+        <v/>
+      </c>
+      <c r="I59" s="6">
+        <f>IF(H59=0,"",G59/H59)</f>
+        <v/>
+      </c>
+      <c r="J59" s="6">
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!BD$5:BD$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="top")*(Marks!BD$5:BD$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="top")*ISNUMBER(Marks!BD$5:BD$39)))</f>
+        <v/>
+      </c>
+      <c r="K59" s="6">
+        <f>IF(SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!BD$5:BD$39))=0,"",SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*(Marks!BD$5:BD$39=1))/SUMPRODUCT((Marks!$BG$5:$BG$39="bottom")*ISNUMBER(Marks!BD$5:BD$39)))</f>
+        <v/>
+      </c>
+      <c r="L59" s="6">
+        <f>IF(OR(J59="",K59=""),"",J59-K59)</f>
+        <v/>
+      </c>
+      <c r="M59">
+        <f>IF(H59=0,"",IF(I59&lt;0.2,"Check the item: fewer than one in five got it right",IF(AND(L59&lt;&gt;"",N(L59)&lt;0),"Check the item: the bottom third beat the top third","")))</f>
+        <v/>
+      </c>
+      <c r="N59">
+        <f>IF(H59=0,"",I59+ROW()/1000000)</f>
         <v/>
       </c>
     </row>
@@ -6869,7 +7193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="6" max="6"/>
@@ -6884,7 +7208,7 @@
     </row>
     <row r="2">
       <c r="B2">
-        <f>IF(SUM(Items!H5:H56)=0,"No marks entered yet.","Most-missed first: take the items from the top.")</f>
+        <f>IF(SUM(Items!H5:H59)=0,"No marks entered yet.","Most-missed first: take the items from the top.")</f>
         <v/>
       </c>
     </row>
@@ -6925,23 +7249,23 @@
         <v>1</v>
       </c>
       <c r="B5">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A5,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A5),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A5,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A5),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C5" s="6">
-        <f>IF(B5="","",INDEX(Items!$I$5:$I$56,MATCH(B5,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B5="","",INDEX(Items!$I$5:$I$59,MATCH(B5,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D5">
-        <f>IF(B5="","",INDEX(Items!$B$5:$B$56,MATCH(B5,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B5="","",INDEX(Items!$B$5:$B$59,MATCH(B5,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E5">
-        <f>IF(B5="","",INDEX(Items!$E$5:$E$56,MATCH(B5,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B5="","",INDEX(Items!$E$5:$E$59,MATCH(B5,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F5">
-        <f>IF(B5="","",INDEX(Items!$M$5:$M$56,MATCH(B5,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B5="","",INDEX(Items!$M$5:$M$59,MATCH(B5,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -6950,23 +7274,23 @@
         <v>2</v>
       </c>
       <c r="B6">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A6,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A6),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A6,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A6),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C6" s="6">
-        <f>IF(B6="","",INDEX(Items!$I$5:$I$56,MATCH(B6,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B6="","",INDEX(Items!$I$5:$I$59,MATCH(B6,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D6">
-        <f>IF(B6="","",INDEX(Items!$B$5:$B$56,MATCH(B6,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B6="","",INDEX(Items!$B$5:$B$59,MATCH(B6,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E6">
-        <f>IF(B6="","",INDEX(Items!$E$5:$E$56,MATCH(B6,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B6="","",INDEX(Items!$E$5:$E$59,MATCH(B6,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F6">
-        <f>IF(B6="","",INDEX(Items!$M$5:$M$56,MATCH(B6,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B6="","",INDEX(Items!$M$5:$M$59,MATCH(B6,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -6975,23 +7299,23 @@
         <v>3</v>
       </c>
       <c r="B7">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A7,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A7),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A7,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A7),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>IF(B7="","",INDEX(Items!$I$5:$I$56,MATCH(B7,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B7="","",INDEX(Items!$I$5:$I$59,MATCH(B7,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D7">
-        <f>IF(B7="","",INDEX(Items!$B$5:$B$56,MATCH(B7,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B7="","",INDEX(Items!$B$5:$B$59,MATCH(B7,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E7">
-        <f>IF(B7="","",INDEX(Items!$E$5:$E$56,MATCH(B7,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B7="","",INDEX(Items!$E$5:$E$59,MATCH(B7,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F7">
-        <f>IF(B7="","",INDEX(Items!$M$5:$M$56,MATCH(B7,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B7="","",INDEX(Items!$M$5:$M$59,MATCH(B7,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7000,23 +7324,23 @@
         <v>4</v>
       </c>
       <c r="B8">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A8,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A8),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A8,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A8),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C8" s="6">
-        <f>IF(B8="","",INDEX(Items!$I$5:$I$56,MATCH(B8,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B8="","",INDEX(Items!$I$5:$I$59,MATCH(B8,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D8">
-        <f>IF(B8="","",INDEX(Items!$B$5:$B$56,MATCH(B8,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B8="","",INDEX(Items!$B$5:$B$59,MATCH(B8,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E8">
-        <f>IF(B8="","",INDEX(Items!$E$5:$E$56,MATCH(B8,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B8="","",INDEX(Items!$E$5:$E$59,MATCH(B8,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F8">
-        <f>IF(B8="","",INDEX(Items!$M$5:$M$56,MATCH(B8,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B8="","",INDEX(Items!$M$5:$M$59,MATCH(B8,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7025,23 +7349,23 @@
         <v>5</v>
       </c>
       <c r="B9">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A9,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A9),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A9,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A9),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C9" s="6">
-        <f>IF(B9="","",INDEX(Items!$I$5:$I$56,MATCH(B9,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B9="","",INDEX(Items!$I$5:$I$59,MATCH(B9,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D9">
-        <f>IF(B9="","",INDEX(Items!$B$5:$B$56,MATCH(B9,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B9="","",INDEX(Items!$B$5:$B$59,MATCH(B9,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E9">
-        <f>IF(B9="","",INDEX(Items!$E$5:$E$56,MATCH(B9,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B9="","",INDEX(Items!$E$5:$E$59,MATCH(B9,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F9">
-        <f>IF(B9="","",INDEX(Items!$M$5:$M$56,MATCH(B9,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B9="","",INDEX(Items!$M$5:$M$59,MATCH(B9,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7050,23 +7374,23 @@
         <v>6</v>
       </c>
       <c r="B10">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A10,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A10),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A10,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A10),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C10" s="6">
-        <f>IF(B10="","",INDEX(Items!$I$5:$I$56,MATCH(B10,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B10="","",INDEX(Items!$I$5:$I$59,MATCH(B10,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D10">
-        <f>IF(B10="","",INDEX(Items!$B$5:$B$56,MATCH(B10,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B10="","",INDEX(Items!$B$5:$B$59,MATCH(B10,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E10">
-        <f>IF(B10="","",INDEX(Items!$E$5:$E$56,MATCH(B10,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B10="","",INDEX(Items!$E$5:$E$59,MATCH(B10,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F10">
-        <f>IF(B10="","",INDEX(Items!$M$5:$M$56,MATCH(B10,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B10="","",INDEX(Items!$M$5:$M$59,MATCH(B10,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7075,23 +7399,23 @@
         <v>7</v>
       </c>
       <c r="B11">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A11,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A11),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A11,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A11),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C11" s="6">
-        <f>IF(B11="","",INDEX(Items!$I$5:$I$56,MATCH(B11,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B11="","",INDEX(Items!$I$5:$I$59,MATCH(B11,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D11">
-        <f>IF(B11="","",INDEX(Items!$B$5:$B$56,MATCH(B11,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B11="","",INDEX(Items!$B$5:$B$59,MATCH(B11,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E11">
-        <f>IF(B11="","",INDEX(Items!$E$5:$E$56,MATCH(B11,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B11="","",INDEX(Items!$E$5:$E$59,MATCH(B11,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F11">
-        <f>IF(B11="","",INDEX(Items!$M$5:$M$56,MATCH(B11,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B11="","",INDEX(Items!$M$5:$M$59,MATCH(B11,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7100,23 +7424,23 @@
         <v>8</v>
       </c>
       <c r="B12">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A12,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A12),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A12,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A12),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C12" s="6">
-        <f>IF(B12="","",INDEX(Items!$I$5:$I$56,MATCH(B12,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B12="","",INDEX(Items!$I$5:$I$59,MATCH(B12,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D12">
-        <f>IF(B12="","",INDEX(Items!$B$5:$B$56,MATCH(B12,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B12="","",INDEX(Items!$B$5:$B$59,MATCH(B12,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E12">
-        <f>IF(B12="","",INDEX(Items!$E$5:$E$56,MATCH(B12,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B12="","",INDEX(Items!$E$5:$E$59,MATCH(B12,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F12">
-        <f>IF(B12="","",INDEX(Items!$M$5:$M$56,MATCH(B12,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B12="","",INDEX(Items!$M$5:$M$59,MATCH(B12,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7125,23 +7449,23 @@
         <v>9</v>
       </c>
       <c r="B13">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A13,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A13),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A13,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A13),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C13" s="6">
-        <f>IF(B13="","",INDEX(Items!$I$5:$I$56,MATCH(B13,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B13="","",INDEX(Items!$I$5:$I$59,MATCH(B13,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D13">
-        <f>IF(B13="","",INDEX(Items!$B$5:$B$56,MATCH(B13,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B13="","",INDEX(Items!$B$5:$B$59,MATCH(B13,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E13">
-        <f>IF(B13="","",INDEX(Items!$E$5:$E$56,MATCH(B13,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B13="","",INDEX(Items!$E$5:$E$59,MATCH(B13,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F13">
-        <f>IF(B13="","",INDEX(Items!$M$5:$M$56,MATCH(B13,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B13="","",INDEX(Items!$M$5:$M$59,MATCH(B13,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7150,23 +7474,23 @@
         <v>10</v>
       </c>
       <c r="B14">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A14,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A14),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A14,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A14),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C14" s="6">
-        <f>IF(B14="","",INDEX(Items!$I$5:$I$56,MATCH(B14,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B14="","",INDEX(Items!$I$5:$I$59,MATCH(B14,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D14">
-        <f>IF(B14="","",INDEX(Items!$B$5:$B$56,MATCH(B14,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B14="","",INDEX(Items!$B$5:$B$59,MATCH(B14,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E14">
-        <f>IF(B14="","",INDEX(Items!$E$5:$E$56,MATCH(B14,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B14="","",INDEX(Items!$E$5:$E$59,MATCH(B14,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F14">
-        <f>IF(B14="","",INDEX(Items!$M$5:$M$56,MATCH(B14,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B14="","",INDEX(Items!$M$5:$M$59,MATCH(B14,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7175,23 +7499,23 @@
         <v>11</v>
       </c>
       <c r="B15">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A15,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A15),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A15,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A15),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C15" s="6">
-        <f>IF(B15="","",INDEX(Items!$I$5:$I$56,MATCH(B15,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B15="","",INDEX(Items!$I$5:$I$59,MATCH(B15,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D15">
-        <f>IF(B15="","",INDEX(Items!$B$5:$B$56,MATCH(B15,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B15="","",INDEX(Items!$B$5:$B$59,MATCH(B15,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E15">
-        <f>IF(B15="","",INDEX(Items!$E$5:$E$56,MATCH(B15,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B15="","",INDEX(Items!$E$5:$E$59,MATCH(B15,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F15">
-        <f>IF(B15="","",INDEX(Items!$M$5:$M$56,MATCH(B15,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B15="","",INDEX(Items!$M$5:$M$59,MATCH(B15,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7200,23 +7524,23 @@
         <v>12</v>
       </c>
       <c r="B16">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A16,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A16),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A16,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A16),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C16" s="6">
-        <f>IF(B16="","",INDEX(Items!$I$5:$I$56,MATCH(B16,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B16="","",INDEX(Items!$I$5:$I$59,MATCH(B16,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D16">
-        <f>IF(B16="","",INDEX(Items!$B$5:$B$56,MATCH(B16,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B16="","",INDEX(Items!$B$5:$B$59,MATCH(B16,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E16">
-        <f>IF(B16="","",INDEX(Items!$E$5:$E$56,MATCH(B16,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B16="","",INDEX(Items!$E$5:$E$59,MATCH(B16,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F16">
-        <f>IF(B16="","",INDEX(Items!$M$5:$M$56,MATCH(B16,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B16="","",INDEX(Items!$M$5:$M$59,MATCH(B16,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7225,23 +7549,23 @@
         <v>13</v>
       </c>
       <c r="B17">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A17,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A17),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A17,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A17),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C17" s="6">
-        <f>IF(B17="","",INDEX(Items!$I$5:$I$56,MATCH(B17,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B17="","",INDEX(Items!$I$5:$I$59,MATCH(B17,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D17">
-        <f>IF(B17="","",INDEX(Items!$B$5:$B$56,MATCH(B17,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B17="","",INDEX(Items!$B$5:$B$59,MATCH(B17,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E17">
-        <f>IF(B17="","",INDEX(Items!$E$5:$E$56,MATCH(B17,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B17="","",INDEX(Items!$E$5:$E$59,MATCH(B17,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F17">
-        <f>IF(B17="","",INDEX(Items!$M$5:$M$56,MATCH(B17,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B17="","",INDEX(Items!$M$5:$M$59,MATCH(B17,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7250,23 +7574,23 @@
         <v>14</v>
       </c>
       <c r="B18">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A18,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A18),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A18,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A18),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C18" s="6">
-        <f>IF(B18="","",INDEX(Items!$I$5:$I$56,MATCH(B18,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B18="","",INDEX(Items!$I$5:$I$59,MATCH(B18,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D18">
-        <f>IF(B18="","",INDEX(Items!$B$5:$B$56,MATCH(B18,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B18="","",INDEX(Items!$B$5:$B$59,MATCH(B18,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E18">
-        <f>IF(B18="","",INDEX(Items!$E$5:$E$56,MATCH(B18,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B18="","",INDEX(Items!$E$5:$E$59,MATCH(B18,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F18">
-        <f>IF(B18="","",INDEX(Items!$M$5:$M$56,MATCH(B18,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B18="","",INDEX(Items!$M$5:$M$59,MATCH(B18,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7275,23 +7599,23 @@
         <v>15</v>
       </c>
       <c r="B19">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A19,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A19),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A19,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A19),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C19" s="6">
-        <f>IF(B19="","",INDEX(Items!$I$5:$I$56,MATCH(B19,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B19="","",INDEX(Items!$I$5:$I$59,MATCH(B19,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D19">
-        <f>IF(B19="","",INDEX(Items!$B$5:$B$56,MATCH(B19,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B19="","",INDEX(Items!$B$5:$B$59,MATCH(B19,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E19">
-        <f>IF(B19="","",INDEX(Items!$E$5:$E$56,MATCH(B19,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B19="","",INDEX(Items!$E$5:$E$59,MATCH(B19,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F19">
-        <f>IF(B19="","",INDEX(Items!$M$5:$M$56,MATCH(B19,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B19="","",INDEX(Items!$M$5:$M$59,MATCH(B19,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7300,23 +7624,23 @@
         <v>16</v>
       </c>
       <c r="B20">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A20,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A20),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A20,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A20),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C20" s="6">
-        <f>IF(B20="","",INDEX(Items!$I$5:$I$56,MATCH(B20,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B20="","",INDEX(Items!$I$5:$I$59,MATCH(B20,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D20">
-        <f>IF(B20="","",INDEX(Items!$B$5:$B$56,MATCH(B20,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B20="","",INDEX(Items!$B$5:$B$59,MATCH(B20,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E20">
-        <f>IF(B20="","",INDEX(Items!$E$5:$E$56,MATCH(B20,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B20="","",INDEX(Items!$E$5:$E$59,MATCH(B20,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F20">
-        <f>IF(B20="","",INDEX(Items!$M$5:$M$56,MATCH(B20,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B20="","",INDEX(Items!$M$5:$M$59,MATCH(B20,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7325,23 +7649,23 @@
         <v>17</v>
       </c>
       <c r="B21">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A21,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A21),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A21,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A21),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C21" s="6">
-        <f>IF(B21="","",INDEX(Items!$I$5:$I$56,MATCH(B21,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B21="","",INDEX(Items!$I$5:$I$59,MATCH(B21,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D21">
-        <f>IF(B21="","",INDEX(Items!$B$5:$B$56,MATCH(B21,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B21="","",INDEX(Items!$B$5:$B$59,MATCH(B21,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E21">
-        <f>IF(B21="","",INDEX(Items!$E$5:$E$56,MATCH(B21,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B21="","",INDEX(Items!$E$5:$E$59,MATCH(B21,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F21">
-        <f>IF(B21="","",INDEX(Items!$M$5:$M$56,MATCH(B21,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B21="","",INDEX(Items!$M$5:$M$59,MATCH(B21,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7350,23 +7674,23 @@
         <v>18</v>
       </c>
       <c r="B22">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A22,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A22),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A22,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A22),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C22" s="6">
-        <f>IF(B22="","",INDEX(Items!$I$5:$I$56,MATCH(B22,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B22="","",INDEX(Items!$I$5:$I$59,MATCH(B22,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D22">
-        <f>IF(B22="","",INDEX(Items!$B$5:$B$56,MATCH(B22,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B22="","",INDEX(Items!$B$5:$B$59,MATCH(B22,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E22">
-        <f>IF(B22="","",INDEX(Items!$E$5:$E$56,MATCH(B22,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B22="","",INDEX(Items!$E$5:$E$59,MATCH(B22,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F22">
-        <f>IF(B22="","",INDEX(Items!$M$5:$M$56,MATCH(B22,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B22="","",INDEX(Items!$M$5:$M$59,MATCH(B22,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7375,23 +7699,23 @@
         <v>19</v>
       </c>
       <c r="B23">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A23,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A23),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A23,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A23),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C23" s="6">
-        <f>IF(B23="","",INDEX(Items!$I$5:$I$56,MATCH(B23,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B23="","",INDEX(Items!$I$5:$I$59,MATCH(B23,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D23">
-        <f>IF(B23="","",INDEX(Items!$B$5:$B$56,MATCH(B23,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B23="","",INDEX(Items!$B$5:$B$59,MATCH(B23,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E23">
-        <f>IF(B23="","",INDEX(Items!$E$5:$E$56,MATCH(B23,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B23="","",INDEX(Items!$E$5:$E$59,MATCH(B23,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F23">
-        <f>IF(B23="","",INDEX(Items!$M$5:$M$56,MATCH(B23,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B23="","",INDEX(Items!$M$5:$M$59,MATCH(B23,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7400,23 +7724,23 @@
         <v>20</v>
       </c>
       <c r="B24">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A24,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A24),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A24,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A24),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C24" s="6">
-        <f>IF(B24="","",INDEX(Items!$I$5:$I$56,MATCH(B24,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B24="","",INDEX(Items!$I$5:$I$59,MATCH(B24,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D24">
-        <f>IF(B24="","",INDEX(Items!$B$5:$B$56,MATCH(B24,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B24="","",INDEX(Items!$B$5:$B$59,MATCH(B24,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E24">
-        <f>IF(B24="","",INDEX(Items!$E$5:$E$56,MATCH(B24,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B24="","",INDEX(Items!$E$5:$E$59,MATCH(B24,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F24">
-        <f>IF(B24="","",INDEX(Items!$M$5:$M$56,MATCH(B24,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B24="","",INDEX(Items!$M$5:$M$59,MATCH(B24,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7425,23 +7749,23 @@
         <v>21</v>
       </c>
       <c r="B25">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A25,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A25),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A25,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A25),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C25" s="6">
-        <f>IF(B25="","",INDEX(Items!$I$5:$I$56,MATCH(B25,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B25="","",INDEX(Items!$I$5:$I$59,MATCH(B25,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D25">
-        <f>IF(B25="","",INDEX(Items!$B$5:$B$56,MATCH(B25,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B25="","",INDEX(Items!$B$5:$B$59,MATCH(B25,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E25">
-        <f>IF(B25="","",INDEX(Items!$E$5:$E$56,MATCH(B25,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B25="","",INDEX(Items!$E$5:$E$59,MATCH(B25,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F25">
-        <f>IF(B25="","",INDEX(Items!$M$5:$M$56,MATCH(B25,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B25="","",INDEX(Items!$M$5:$M$59,MATCH(B25,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7450,23 +7774,23 @@
         <v>22</v>
       </c>
       <c r="B26">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A26,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A26),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A26,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A26),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C26" s="6">
-        <f>IF(B26="","",INDEX(Items!$I$5:$I$56,MATCH(B26,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B26="","",INDEX(Items!$I$5:$I$59,MATCH(B26,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D26">
-        <f>IF(B26="","",INDEX(Items!$B$5:$B$56,MATCH(B26,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B26="","",INDEX(Items!$B$5:$B$59,MATCH(B26,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E26">
-        <f>IF(B26="","",INDEX(Items!$E$5:$E$56,MATCH(B26,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B26="","",INDEX(Items!$E$5:$E$59,MATCH(B26,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F26">
-        <f>IF(B26="","",INDEX(Items!$M$5:$M$56,MATCH(B26,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B26="","",INDEX(Items!$M$5:$M$59,MATCH(B26,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7475,23 +7799,23 @@
         <v>23</v>
       </c>
       <c r="B27">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A27,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A27),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A27,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A27),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C27" s="6">
-        <f>IF(B27="","",INDEX(Items!$I$5:$I$56,MATCH(B27,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B27="","",INDEX(Items!$I$5:$I$59,MATCH(B27,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D27">
-        <f>IF(B27="","",INDEX(Items!$B$5:$B$56,MATCH(B27,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B27="","",INDEX(Items!$B$5:$B$59,MATCH(B27,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E27">
-        <f>IF(B27="","",INDEX(Items!$E$5:$E$56,MATCH(B27,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B27="","",INDEX(Items!$E$5:$E$59,MATCH(B27,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F27">
-        <f>IF(B27="","",INDEX(Items!$M$5:$M$56,MATCH(B27,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B27="","",INDEX(Items!$M$5:$M$59,MATCH(B27,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7500,23 +7824,23 @@
         <v>24</v>
       </c>
       <c r="B28">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A28,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A28),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A28,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A28),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C28" s="6">
-        <f>IF(B28="","",INDEX(Items!$I$5:$I$56,MATCH(B28,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B28="","",INDEX(Items!$I$5:$I$59,MATCH(B28,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D28">
-        <f>IF(B28="","",INDEX(Items!$B$5:$B$56,MATCH(B28,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B28="","",INDEX(Items!$B$5:$B$59,MATCH(B28,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E28">
-        <f>IF(B28="","",INDEX(Items!$E$5:$E$56,MATCH(B28,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B28="","",INDEX(Items!$E$5:$E$59,MATCH(B28,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F28">
-        <f>IF(B28="","",INDEX(Items!$M$5:$M$56,MATCH(B28,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B28="","",INDEX(Items!$M$5:$M$59,MATCH(B28,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7525,23 +7849,23 @@
         <v>25</v>
       </c>
       <c r="B29">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A29,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A29),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A29,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A29),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C29" s="6">
-        <f>IF(B29="","",INDEX(Items!$I$5:$I$56,MATCH(B29,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B29="","",INDEX(Items!$I$5:$I$59,MATCH(B29,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D29">
-        <f>IF(B29="","",INDEX(Items!$B$5:$B$56,MATCH(B29,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B29="","",INDEX(Items!$B$5:$B$59,MATCH(B29,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E29">
-        <f>IF(B29="","",INDEX(Items!$E$5:$E$56,MATCH(B29,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B29="","",INDEX(Items!$E$5:$E$59,MATCH(B29,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F29">
-        <f>IF(B29="","",INDEX(Items!$M$5:$M$56,MATCH(B29,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B29="","",INDEX(Items!$M$5:$M$59,MATCH(B29,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7550,23 +7874,23 @@
         <v>26</v>
       </c>
       <c r="B30">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A30,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A30),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A30,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A30),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C30" s="6">
-        <f>IF(B30="","",INDEX(Items!$I$5:$I$56,MATCH(B30,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B30="","",INDEX(Items!$I$5:$I$59,MATCH(B30,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D30">
-        <f>IF(B30="","",INDEX(Items!$B$5:$B$56,MATCH(B30,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B30="","",INDEX(Items!$B$5:$B$59,MATCH(B30,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E30">
-        <f>IF(B30="","",INDEX(Items!$E$5:$E$56,MATCH(B30,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B30="","",INDEX(Items!$E$5:$E$59,MATCH(B30,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F30">
-        <f>IF(B30="","",INDEX(Items!$M$5:$M$56,MATCH(B30,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B30="","",INDEX(Items!$M$5:$M$59,MATCH(B30,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7575,23 +7899,23 @@
         <v>27</v>
       </c>
       <c r="B31">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A31,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A31),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A31,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A31),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C31" s="6">
-        <f>IF(B31="","",INDEX(Items!$I$5:$I$56,MATCH(B31,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B31="","",INDEX(Items!$I$5:$I$59,MATCH(B31,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D31">
-        <f>IF(B31="","",INDEX(Items!$B$5:$B$56,MATCH(B31,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B31="","",INDEX(Items!$B$5:$B$59,MATCH(B31,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E31">
-        <f>IF(B31="","",INDEX(Items!$E$5:$E$56,MATCH(B31,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B31="","",INDEX(Items!$E$5:$E$59,MATCH(B31,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F31">
-        <f>IF(B31="","",INDEX(Items!$M$5:$M$56,MATCH(B31,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B31="","",INDEX(Items!$M$5:$M$59,MATCH(B31,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7600,23 +7924,23 @@
         <v>28</v>
       </c>
       <c r="B32">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A32,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A32),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A32,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A32),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C32" s="6">
-        <f>IF(B32="","",INDEX(Items!$I$5:$I$56,MATCH(B32,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B32="","",INDEX(Items!$I$5:$I$59,MATCH(B32,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D32">
-        <f>IF(B32="","",INDEX(Items!$B$5:$B$56,MATCH(B32,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B32="","",INDEX(Items!$B$5:$B$59,MATCH(B32,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E32">
-        <f>IF(B32="","",INDEX(Items!$E$5:$E$56,MATCH(B32,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B32="","",INDEX(Items!$E$5:$E$59,MATCH(B32,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F32">
-        <f>IF(B32="","",INDEX(Items!$M$5:$M$56,MATCH(B32,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B32="","",INDEX(Items!$M$5:$M$59,MATCH(B32,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7625,23 +7949,23 @@
         <v>29</v>
       </c>
       <c r="B33">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A33,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A33),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A33,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A33),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C33" s="6">
-        <f>IF(B33="","",INDEX(Items!$I$5:$I$56,MATCH(B33,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B33="","",INDEX(Items!$I$5:$I$59,MATCH(B33,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D33">
-        <f>IF(B33="","",INDEX(Items!$B$5:$B$56,MATCH(B33,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B33="","",INDEX(Items!$B$5:$B$59,MATCH(B33,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E33">
-        <f>IF(B33="","",INDEX(Items!$E$5:$E$56,MATCH(B33,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B33="","",INDEX(Items!$E$5:$E$59,MATCH(B33,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F33">
-        <f>IF(B33="","",INDEX(Items!$M$5:$M$56,MATCH(B33,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B33="","",INDEX(Items!$M$5:$M$59,MATCH(B33,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7650,23 +7974,23 @@
         <v>30</v>
       </c>
       <c r="B34">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A34,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A34),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A34,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A34),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C34" s="6">
-        <f>IF(B34="","",INDEX(Items!$I$5:$I$56,MATCH(B34,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B34="","",INDEX(Items!$I$5:$I$59,MATCH(B34,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D34">
-        <f>IF(B34="","",INDEX(Items!$B$5:$B$56,MATCH(B34,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B34="","",INDEX(Items!$B$5:$B$59,MATCH(B34,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E34">
-        <f>IF(B34="","",INDEX(Items!$E$5:$E$56,MATCH(B34,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B34="","",INDEX(Items!$E$5:$E$59,MATCH(B34,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F34">
-        <f>IF(B34="","",INDEX(Items!$M$5:$M$56,MATCH(B34,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B34="","",INDEX(Items!$M$5:$M$59,MATCH(B34,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7675,23 +7999,23 @@
         <v>31</v>
       </c>
       <c r="B35">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A35,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A35),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A35,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A35),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C35" s="6">
-        <f>IF(B35="","",INDEX(Items!$I$5:$I$56,MATCH(B35,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B35="","",INDEX(Items!$I$5:$I$59,MATCH(B35,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D35">
-        <f>IF(B35="","",INDEX(Items!$B$5:$B$56,MATCH(B35,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B35="","",INDEX(Items!$B$5:$B$59,MATCH(B35,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E35">
-        <f>IF(B35="","",INDEX(Items!$E$5:$E$56,MATCH(B35,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B35="","",INDEX(Items!$E$5:$E$59,MATCH(B35,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F35">
-        <f>IF(B35="","",INDEX(Items!$M$5:$M$56,MATCH(B35,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B35="","",INDEX(Items!$M$5:$M$59,MATCH(B35,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7700,23 +8024,23 @@
         <v>32</v>
       </c>
       <c r="B36">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A36,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A36),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A36,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A36),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C36" s="6">
-        <f>IF(B36="","",INDEX(Items!$I$5:$I$56,MATCH(B36,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B36="","",INDEX(Items!$I$5:$I$59,MATCH(B36,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D36">
-        <f>IF(B36="","",INDEX(Items!$B$5:$B$56,MATCH(B36,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B36="","",INDEX(Items!$B$5:$B$59,MATCH(B36,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E36">
-        <f>IF(B36="","",INDEX(Items!$E$5:$E$56,MATCH(B36,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B36="","",INDEX(Items!$E$5:$E$59,MATCH(B36,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F36">
-        <f>IF(B36="","",INDEX(Items!$M$5:$M$56,MATCH(B36,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B36="","",INDEX(Items!$M$5:$M$59,MATCH(B36,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7725,23 +8049,23 @@
         <v>33</v>
       </c>
       <c r="B37">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A37,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A37),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A37,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A37),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C37" s="6">
-        <f>IF(B37="","",INDEX(Items!$I$5:$I$56,MATCH(B37,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B37="","",INDEX(Items!$I$5:$I$59,MATCH(B37,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D37">
-        <f>IF(B37="","",INDEX(Items!$B$5:$B$56,MATCH(B37,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B37="","",INDEX(Items!$B$5:$B$59,MATCH(B37,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E37">
-        <f>IF(B37="","",INDEX(Items!$E$5:$E$56,MATCH(B37,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B37="","",INDEX(Items!$E$5:$E$59,MATCH(B37,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F37">
-        <f>IF(B37="","",INDEX(Items!$M$5:$M$56,MATCH(B37,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B37="","",INDEX(Items!$M$5:$M$59,MATCH(B37,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7750,23 +8074,23 @@
         <v>34</v>
       </c>
       <c r="B38">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A38,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A38),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A38,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A38),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C38" s="6">
-        <f>IF(B38="","",INDEX(Items!$I$5:$I$56,MATCH(B38,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B38="","",INDEX(Items!$I$5:$I$59,MATCH(B38,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D38">
-        <f>IF(B38="","",INDEX(Items!$B$5:$B$56,MATCH(B38,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B38="","",INDEX(Items!$B$5:$B$59,MATCH(B38,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E38">
-        <f>IF(B38="","",INDEX(Items!$E$5:$E$56,MATCH(B38,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B38="","",INDEX(Items!$E$5:$E$59,MATCH(B38,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F38">
-        <f>IF(B38="","",INDEX(Items!$M$5:$M$56,MATCH(B38,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B38="","",INDEX(Items!$M$5:$M$59,MATCH(B38,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7775,23 +8099,23 @@
         <v>35</v>
       </c>
       <c r="B39">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A39,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A39),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A39,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A39),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C39" s="6">
-        <f>IF(B39="","",INDEX(Items!$I$5:$I$56,MATCH(B39,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B39="","",INDEX(Items!$I$5:$I$59,MATCH(B39,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D39">
-        <f>IF(B39="","",INDEX(Items!$B$5:$B$56,MATCH(B39,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B39="","",INDEX(Items!$B$5:$B$59,MATCH(B39,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E39">
-        <f>IF(B39="","",INDEX(Items!$E$5:$E$56,MATCH(B39,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B39="","",INDEX(Items!$E$5:$E$59,MATCH(B39,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F39">
-        <f>IF(B39="","",INDEX(Items!$M$5:$M$56,MATCH(B39,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B39="","",INDEX(Items!$M$5:$M$59,MATCH(B39,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7800,23 +8124,23 @@
         <v>36</v>
       </c>
       <c r="B40">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A40,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A40),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A40,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A40),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C40" s="6">
-        <f>IF(B40="","",INDEX(Items!$I$5:$I$56,MATCH(B40,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B40="","",INDEX(Items!$I$5:$I$59,MATCH(B40,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D40">
-        <f>IF(B40="","",INDEX(Items!$B$5:$B$56,MATCH(B40,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B40="","",INDEX(Items!$B$5:$B$59,MATCH(B40,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E40">
-        <f>IF(B40="","",INDEX(Items!$E$5:$E$56,MATCH(B40,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B40="","",INDEX(Items!$E$5:$E$59,MATCH(B40,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F40">
-        <f>IF(B40="","",INDEX(Items!$M$5:$M$56,MATCH(B40,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B40="","",INDEX(Items!$M$5:$M$59,MATCH(B40,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7825,23 +8149,23 @@
         <v>37</v>
       </c>
       <c r="B41">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A41,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A41),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A41,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A41),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C41" s="6">
-        <f>IF(B41="","",INDEX(Items!$I$5:$I$56,MATCH(B41,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B41="","",INDEX(Items!$I$5:$I$59,MATCH(B41,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D41">
-        <f>IF(B41="","",INDEX(Items!$B$5:$B$56,MATCH(B41,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B41="","",INDEX(Items!$B$5:$B$59,MATCH(B41,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E41">
-        <f>IF(B41="","",INDEX(Items!$E$5:$E$56,MATCH(B41,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B41="","",INDEX(Items!$E$5:$E$59,MATCH(B41,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F41">
-        <f>IF(B41="","",INDEX(Items!$M$5:$M$56,MATCH(B41,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B41="","",INDEX(Items!$M$5:$M$59,MATCH(B41,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7850,23 +8174,23 @@
         <v>38</v>
       </c>
       <c r="B42">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A42,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A42),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A42,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A42),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C42" s="6">
-        <f>IF(B42="","",INDEX(Items!$I$5:$I$56,MATCH(B42,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B42="","",INDEX(Items!$I$5:$I$59,MATCH(B42,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D42">
-        <f>IF(B42="","",INDEX(Items!$B$5:$B$56,MATCH(B42,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B42="","",INDEX(Items!$B$5:$B$59,MATCH(B42,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E42">
-        <f>IF(B42="","",INDEX(Items!$E$5:$E$56,MATCH(B42,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B42="","",INDEX(Items!$E$5:$E$59,MATCH(B42,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F42">
-        <f>IF(B42="","",INDEX(Items!$M$5:$M$56,MATCH(B42,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B42="","",INDEX(Items!$M$5:$M$59,MATCH(B42,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7875,23 +8199,23 @@
         <v>39</v>
       </c>
       <c r="B43">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A43,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A43),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A43,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A43),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C43" s="6">
-        <f>IF(B43="","",INDEX(Items!$I$5:$I$56,MATCH(B43,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B43="","",INDEX(Items!$I$5:$I$59,MATCH(B43,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D43">
-        <f>IF(B43="","",INDEX(Items!$B$5:$B$56,MATCH(B43,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B43="","",INDEX(Items!$B$5:$B$59,MATCH(B43,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E43">
-        <f>IF(B43="","",INDEX(Items!$E$5:$E$56,MATCH(B43,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B43="","",INDEX(Items!$E$5:$E$59,MATCH(B43,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F43">
-        <f>IF(B43="","",INDEX(Items!$M$5:$M$56,MATCH(B43,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B43="","",INDEX(Items!$M$5:$M$59,MATCH(B43,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7900,23 +8224,23 @@
         <v>40</v>
       </c>
       <c r="B44">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A44,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A44),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A44,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A44),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C44" s="6">
-        <f>IF(B44="","",INDEX(Items!$I$5:$I$56,MATCH(B44,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B44="","",INDEX(Items!$I$5:$I$59,MATCH(B44,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D44">
-        <f>IF(B44="","",INDEX(Items!$B$5:$B$56,MATCH(B44,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B44="","",INDEX(Items!$B$5:$B$59,MATCH(B44,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E44">
-        <f>IF(B44="","",INDEX(Items!$E$5:$E$56,MATCH(B44,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B44="","",INDEX(Items!$E$5:$E$59,MATCH(B44,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F44">
-        <f>IF(B44="","",INDEX(Items!$M$5:$M$56,MATCH(B44,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B44="","",INDEX(Items!$M$5:$M$59,MATCH(B44,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7925,23 +8249,23 @@
         <v>41</v>
       </c>
       <c r="B45">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A45,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A45),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A45,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A45),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C45" s="6">
-        <f>IF(B45="","",INDEX(Items!$I$5:$I$56,MATCH(B45,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B45="","",INDEX(Items!$I$5:$I$59,MATCH(B45,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D45">
-        <f>IF(B45="","",INDEX(Items!$B$5:$B$56,MATCH(B45,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B45="","",INDEX(Items!$B$5:$B$59,MATCH(B45,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E45">
-        <f>IF(B45="","",INDEX(Items!$E$5:$E$56,MATCH(B45,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B45="","",INDEX(Items!$E$5:$E$59,MATCH(B45,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F45">
-        <f>IF(B45="","",INDEX(Items!$M$5:$M$56,MATCH(B45,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B45="","",INDEX(Items!$M$5:$M$59,MATCH(B45,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7950,23 +8274,23 @@
         <v>42</v>
       </c>
       <c r="B46">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A46,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A46),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A46,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A46),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C46" s="6">
-        <f>IF(B46="","",INDEX(Items!$I$5:$I$56,MATCH(B46,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B46="","",INDEX(Items!$I$5:$I$59,MATCH(B46,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D46">
-        <f>IF(B46="","",INDEX(Items!$B$5:$B$56,MATCH(B46,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B46="","",INDEX(Items!$B$5:$B$59,MATCH(B46,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E46">
-        <f>IF(B46="","",INDEX(Items!$E$5:$E$56,MATCH(B46,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B46="","",INDEX(Items!$E$5:$E$59,MATCH(B46,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F46">
-        <f>IF(B46="","",INDEX(Items!$M$5:$M$56,MATCH(B46,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B46="","",INDEX(Items!$M$5:$M$59,MATCH(B46,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -7975,23 +8299,23 @@
         <v>43</v>
       </c>
       <c r="B47">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A47,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A47),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A47,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A47),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C47" s="6">
-        <f>IF(B47="","",INDEX(Items!$I$5:$I$56,MATCH(B47,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B47="","",INDEX(Items!$I$5:$I$59,MATCH(B47,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D47">
-        <f>IF(B47="","",INDEX(Items!$B$5:$B$56,MATCH(B47,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B47="","",INDEX(Items!$B$5:$B$59,MATCH(B47,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E47">
-        <f>IF(B47="","",INDEX(Items!$E$5:$E$56,MATCH(B47,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B47="","",INDEX(Items!$E$5:$E$59,MATCH(B47,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F47">
-        <f>IF(B47="","",INDEX(Items!$M$5:$M$56,MATCH(B47,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B47="","",INDEX(Items!$M$5:$M$59,MATCH(B47,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -8000,23 +8324,23 @@
         <v>44</v>
       </c>
       <c r="B48">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A48,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A48),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A48,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A48),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C48" s="6">
-        <f>IF(B48="","",INDEX(Items!$I$5:$I$56,MATCH(B48,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B48="","",INDEX(Items!$I$5:$I$59,MATCH(B48,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D48">
-        <f>IF(B48="","",INDEX(Items!$B$5:$B$56,MATCH(B48,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B48="","",INDEX(Items!$B$5:$B$59,MATCH(B48,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E48">
-        <f>IF(B48="","",INDEX(Items!$E$5:$E$56,MATCH(B48,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B48="","",INDEX(Items!$E$5:$E$59,MATCH(B48,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F48">
-        <f>IF(B48="","",INDEX(Items!$M$5:$M$56,MATCH(B48,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B48="","",INDEX(Items!$M$5:$M$59,MATCH(B48,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -8025,23 +8349,23 @@
         <v>45</v>
       </c>
       <c r="B49">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A49,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A49),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A49,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A49),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C49" s="6">
-        <f>IF(B49="","",INDEX(Items!$I$5:$I$56,MATCH(B49,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B49="","",INDEX(Items!$I$5:$I$59,MATCH(B49,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D49">
-        <f>IF(B49="","",INDEX(Items!$B$5:$B$56,MATCH(B49,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B49="","",INDEX(Items!$B$5:$B$59,MATCH(B49,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E49">
-        <f>IF(B49="","",INDEX(Items!$E$5:$E$56,MATCH(B49,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B49="","",INDEX(Items!$E$5:$E$59,MATCH(B49,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F49">
-        <f>IF(B49="","",INDEX(Items!$M$5:$M$56,MATCH(B49,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B49="","",INDEX(Items!$M$5:$M$59,MATCH(B49,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -8050,23 +8374,23 @@
         <v>46</v>
       </c>
       <c r="B50">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A50,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A50),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A50,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A50),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C50" s="6">
-        <f>IF(B50="","",INDEX(Items!$I$5:$I$56,MATCH(B50,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B50="","",INDEX(Items!$I$5:$I$59,MATCH(B50,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D50">
-        <f>IF(B50="","",INDEX(Items!$B$5:$B$56,MATCH(B50,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B50="","",INDEX(Items!$B$5:$B$59,MATCH(B50,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E50">
-        <f>IF(B50="","",INDEX(Items!$E$5:$E$56,MATCH(B50,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B50="","",INDEX(Items!$E$5:$E$59,MATCH(B50,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F50">
-        <f>IF(B50="","",INDEX(Items!$M$5:$M$56,MATCH(B50,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B50="","",INDEX(Items!$M$5:$M$59,MATCH(B50,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -8075,23 +8399,23 @@
         <v>47</v>
       </c>
       <c r="B51">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A51,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A51),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A51,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A51),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C51" s="6">
-        <f>IF(B51="","",INDEX(Items!$I$5:$I$56,MATCH(B51,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B51="","",INDEX(Items!$I$5:$I$59,MATCH(B51,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D51">
-        <f>IF(B51="","",INDEX(Items!$B$5:$B$56,MATCH(B51,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B51="","",INDEX(Items!$B$5:$B$59,MATCH(B51,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E51">
-        <f>IF(B51="","",INDEX(Items!$E$5:$E$56,MATCH(B51,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B51="","",INDEX(Items!$E$5:$E$59,MATCH(B51,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F51">
-        <f>IF(B51="","",INDEX(Items!$M$5:$M$56,MATCH(B51,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B51="","",INDEX(Items!$M$5:$M$59,MATCH(B51,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -8100,23 +8424,23 @@
         <v>48</v>
       </c>
       <c r="B52">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A52,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A52),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A52,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A52),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C52" s="6">
-        <f>IF(B52="","",INDEX(Items!$I$5:$I$56,MATCH(B52,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B52="","",INDEX(Items!$I$5:$I$59,MATCH(B52,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D52">
-        <f>IF(B52="","",INDEX(Items!$B$5:$B$56,MATCH(B52,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B52="","",INDEX(Items!$B$5:$B$59,MATCH(B52,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E52">
-        <f>IF(B52="","",INDEX(Items!$E$5:$E$56,MATCH(B52,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B52="","",INDEX(Items!$E$5:$E$59,MATCH(B52,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F52">
-        <f>IF(B52="","",INDEX(Items!$M$5:$M$56,MATCH(B52,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B52="","",INDEX(Items!$M$5:$M$59,MATCH(B52,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -8125,23 +8449,23 @@
         <v>49</v>
       </c>
       <c r="B53">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A53,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A53),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A53,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A53),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C53" s="6">
-        <f>IF(B53="","",INDEX(Items!$I$5:$I$56,MATCH(B53,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B53="","",INDEX(Items!$I$5:$I$59,MATCH(B53,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D53">
-        <f>IF(B53="","",INDEX(Items!$B$5:$B$56,MATCH(B53,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B53="","",INDEX(Items!$B$5:$B$59,MATCH(B53,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E53">
-        <f>IF(B53="","",INDEX(Items!$E$5:$E$56,MATCH(B53,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B53="","",INDEX(Items!$E$5:$E$59,MATCH(B53,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F53">
-        <f>IF(B53="","",INDEX(Items!$M$5:$M$56,MATCH(B53,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B53="","",INDEX(Items!$M$5:$M$59,MATCH(B53,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -8150,23 +8474,23 @@
         <v>50</v>
       </c>
       <c r="B54">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A54,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A54),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A54,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A54),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C54" s="6">
-        <f>IF(B54="","",INDEX(Items!$I$5:$I$56,MATCH(B54,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B54="","",INDEX(Items!$I$5:$I$59,MATCH(B54,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D54">
-        <f>IF(B54="","",INDEX(Items!$B$5:$B$56,MATCH(B54,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B54="","",INDEX(Items!$B$5:$B$59,MATCH(B54,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E54">
-        <f>IF(B54="","",INDEX(Items!$E$5:$E$56,MATCH(B54,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B54="","",INDEX(Items!$E$5:$E$59,MATCH(B54,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F54">
-        <f>IF(B54="","",INDEX(Items!$M$5:$M$56,MATCH(B54,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B54="","",INDEX(Items!$M$5:$M$59,MATCH(B54,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -8175,23 +8499,23 @@
         <v>51</v>
       </c>
       <c r="B55">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A55,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A55),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A55,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A55),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C55" s="6">
-        <f>IF(B55="","",INDEX(Items!$I$5:$I$56,MATCH(B55,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B55="","",INDEX(Items!$I$5:$I$59,MATCH(B55,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D55">
-        <f>IF(B55="","",INDEX(Items!$B$5:$B$56,MATCH(B55,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B55="","",INDEX(Items!$B$5:$B$59,MATCH(B55,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E55">
-        <f>IF(B55="","",INDEX(Items!$E$5:$E$56,MATCH(B55,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B55="","",INDEX(Items!$E$5:$E$59,MATCH(B55,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F55">
-        <f>IF(B55="","",INDEX(Items!$M$5:$M$56,MATCH(B55,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B55="","",INDEX(Items!$M$5:$M$59,MATCH(B55,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -8200,23 +8524,98 @@
         <v>52</v>
       </c>
       <c r="B56">
-        <f>IF(COUNT(Items!$N$5:$N$56)&lt;A56,"",INDEX(Items!$A$5:$A$56,MATCH(SMALL(Items!$N$5:$N$56,A56),Items!$N$5:$N$56,0)))</f>
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A56,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A56),Items!$N$5:$N$59,0)))</f>
         <v/>
       </c>
       <c r="C56" s="6">
-        <f>IF(B56="","",INDEX(Items!$I$5:$I$56,MATCH(B56,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B56="","",INDEX(Items!$I$5:$I$59,MATCH(B56,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="D56">
-        <f>IF(B56="","",INDEX(Items!$B$5:$B$56,MATCH(B56,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B56="","",INDEX(Items!$B$5:$B$59,MATCH(B56,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="E56">
-        <f>IF(B56="","",INDEX(Items!$E$5:$E$56,MATCH(B56,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B56="","",INDEX(Items!$E$5:$E$59,MATCH(B56,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
       <c r="F56">
-        <f>IF(B56="","",INDEX(Items!$M$5:$M$56,MATCH(B56,Items!$A$5:$A$56,0)))</f>
+        <f>IF(B56="","",INDEX(Items!$M$5:$M$59,MATCH(B56,Items!$A$5:$A$59,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>53</v>
+      </c>
+      <c r="B57">
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A57,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A57),Items!$N$5:$N$59,0)))</f>
+        <v/>
+      </c>
+      <c r="C57" s="6">
+        <f>IF(B57="","",INDEX(Items!$I$5:$I$59,MATCH(B57,Items!$A$5:$A$59,0)))</f>
+        <v/>
+      </c>
+      <c r="D57">
+        <f>IF(B57="","",INDEX(Items!$B$5:$B$59,MATCH(B57,Items!$A$5:$A$59,0)))</f>
+        <v/>
+      </c>
+      <c r="E57">
+        <f>IF(B57="","",INDEX(Items!$E$5:$E$59,MATCH(B57,Items!$A$5:$A$59,0)))</f>
+        <v/>
+      </c>
+      <c r="F57">
+        <f>IF(B57="","",INDEX(Items!$M$5:$M$59,MATCH(B57,Items!$A$5:$A$59,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>54</v>
+      </c>
+      <c r="B58">
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A58,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A58),Items!$N$5:$N$59,0)))</f>
+        <v/>
+      </c>
+      <c r="C58" s="6">
+        <f>IF(B58="","",INDEX(Items!$I$5:$I$59,MATCH(B58,Items!$A$5:$A$59,0)))</f>
+        <v/>
+      </c>
+      <c r="D58">
+        <f>IF(B58="","",INDEX(Items!$B$5:$B$59,MATCH(B58,Items!$A$5:$A$59,0)))</f>
+        <v/>
+      </c>
+      <c r="E58">
+        <f>IF(B58="","",INDEX(Items!$E$5:$E$59,MATCH(B58,Items!$A$5:$A$59,0)))</f>
+        <v/>
+      </c>
+      <c r="F58">
+        <f>IF(B58="","",INDEX(Items!$M$5:$M$59,MATCH(B58,Items!$A$5:$A$59,0)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>55</v>
+      </c>
+      <c r="B59">
+        <f>IF(COUNT(Items!$N$5:$N$59)&lt;A59,"",INDEX(Items!$A$5:$A$59,MATCH(SMALL(Items!$N$5:$N$59,A59),Items!$N$5:$N$59,0)))</f>
+        <v/>
+      </c>
+      <c r="C59" s="6">
+        <f>IF(B59="","",INDEX(Items!$I$5:$I$59,MATCH(B59,Items!$A$5:$A$59,0)))</f>
+        <v/>
+      </c>
+      <c r="D59">
+        <f>IF(B59="","",INDEX(Items!$B$5:$B$59,MATCH(B59,Items!$A$5:$A$59,0)))</f>
+        <v/>
+      </c>
+      <c r="E59">
+        <f>IF(B59="","",INDEX(Items!$E$5:$E$59,MATCH(B59,Items!$A$5:$A$59,0)))</f>
+        <v/>
+      </c>
+      <c r="F59">
+        <f>IF(B59="","",INDEX(Items!$M$5:$M$59,MATCH(B59,Items!$A$5:$A$59,0)))</f>
         <v/>
       </c>
     </row>
@@ -8278,11 +8677,11 @@
         </is>
       </c>
       <c r="C5">
-        <f>COUNTIF(Items!$E$5:$E$56,A5)</f>
+        <f>COUNTIF(Items!$E$5:$E$59,A5)</f>
         <v/>
       </c>
       <c r="D5" s="6">
-        <f>IF(SUMPRODUCT((Items!$E$5:$E$56=A5)*Items!$H$5:$H$56)=0,"",SUMPRODUCT((Items!$E$5:$E$56=A5)*Items!$G$5:$G$56)/SUMPRODUCT((Items!$E$5:$E$56=A5)*Items!$H$5:$H$56))</f>
+        <f>IF(SUMPRODUCT((Items!$E$5:$E$59=A5)*Items!$H$5:$H$59)=0,"",SUMPRODUCT((Items!$E$5:$E$59=A5)*Items!$G$5:$G$59)/SUMPRODUCT((Items!$E$5:$E$59=A5)*Items!$H$5:$H$59))</f>
         <v/>
       </c>
     </row>
@@ -8298,11 +8697,11 @@
         </is>
       </c>
       <c r="C6">
-        <f>COUNTIF(Items!$E$5:$E$56,A6)</f>
+        <f>COUNTIF(Items!$E$5:$E$59,A6)</f>
         <v/>
       </c>
       <c r="D6" s="6">
-        <f>IF(SUMPRODUCT((Items!$E$5:$E$56=A6)*Items!$H$5:$H$56)=0,"",SUMPRODUCT((Items!$E$5:$E$56=A6)*Items!$G$5:$G$56)/SUMPRODUCT((Items!$E$5:$E$56=A6)*Items!$H$5:$H$56))</f>
+        <f>IF(SUMPRODUCT((Items!$E$5:$E$59=A6)*Items!$H$5:$H$59)=0,"",SUMPRODUCT((Items!$E$5:$E$59=A6)*Items!$G$5:$G$59)/SUMPRODUCT((Items!$E$5:$E$59=A6)*Items!$H$5:$H$59))</f>
         <v/>
       </c>
     </row>
@@ -8318,11 +8717,11 @@
         </is>
       </c>
       <c r="C7">
-        <f>COUNTIF(Items!$E$5:$E$56,A7)</f>
+        <f>COUNTIF(Items!$E$5:$E$59,A7)</f>
         <v/>
       </c>
       <c r="D7" s="6">
-        <f>IF(SUMPRODUCT((Items!$E$5:$E$56=A7)*Items!$H$5:$H$56)=0,"",SUMPRODUCT((Items!$E$5:$E$56=A7)*Items!$G$5:$G$56)/SUMPRODUCT((Items!$E$5:$E$56=A7)*Items!$H$5:$H$56))</f>
+        <f>IF(SUMPRODUCT((Items!$E$5:$E$59=A7)*Items!$H$5:$H$59)=0,"",SUMPRODUCT((Items!$E$5:$E$59=A7)*Items!$G$5:$G$59)/SUMPRODUCT((Items!$E$5:$E$59=A7)*Items!$H$5:$H$59))</f>
         <v/>
       </c>
     </row>
@@ -8336,11 +8735,11 @@
         </is>
       </c>
       <c r="C8">
-        <f>COUNTIF(Items!$B$5:$B$56,A8)</f>
+        <f>COUNTIF(Items!$B$5:$B$59,A8)</f>
         <v/>
       </c>
       <c r="D8" s="6">
-        <f>IF(SUMPRODUCT((Items!$B$5:$B$56=A8)*Items!$H$5:$H$56)=0,"",SUMPRODUCT((Items!$B$5:$B$56=A8)*Items!$G$5:$G$56)/SUMPRODUCT((Items!$B$5:$B$56=A8)*Items!$H$5:$H$56))</f>
+        <f>IF(SUMPRODUCT((Items!$B$5:$B$59=A8)*Items!$H$5:$H$59)=0,"",SUMPRODUCT((Items!$B$5:$B$59=A8)*Items!$G$5:$G$59)/SUMPRODUCT((Items!$B$5:$B$59=A8)*Items!$H$5:$H$59))</f>
         <v/>
       </c>
     </row>
@@ -8354,11 +8753,11 @@
         </is>
       </c>
       <c r="C9">
-        <f>COUNTIF(Items!$B$5:$B$56,A9)</f>
+        <f>COUNTIF(Items!$B$5:$B$59,A9)</f>
         <v/>
       </c>
       <c r="D9" s="6">
-        <f>IF(SUMPRODUCT((Items!$B$5:$B$56=A9)*Items!$H$5:$H$56)=0,"",SUMPRODUCT((Items!$B$5:$B$56=A9)*Items!$G$5:$G$56)/SUMPRODUCT((Items!$B$5:$B$56=A9)*Items!$H$5:$H$56))</f>
+        <f>IF(SUMPRODUCT((Items!$B$5:$B$59=A9)*Items!$H$5:$H$59)=0,"",SUMPRODUCT((Items!$B$5:$B$59=A9)*Items!$G$5:$G$59)/SUMPRODUCT((Items!$B$5:$B$59=A9)*Items!$H$5:$H$59))</f>
         <v/>
       </c>
     </row>
@@ -8372,11 +8771,11 @@
         </is>
       </c>
       <c r="C10">
-        <f>COUNTIF(Items!$B$5:$B$56,A10)</f>
+        <f>COUNTIF(Items!$B$5:$B$59,A10)</f>
         <v/>
       </c>
       <c r="D10" s="6">
-        <f>IF(SUMPRODUCT((Items!$B$5:$B$56=A10)*Items!$H$5:$H$56)=0,"",SUMPRODUCT((Items!$B$5:$B$56=A10)*Items!$G$5:$G$56)/SUMPRODUCT((Items!$B$5:$B$56=A10)*Items!$H$5:$H$56))</f>
+        <f>IF(SUMPRODUCT((Items!$B$5:$B$59=A10)*Items!$H$5:$H$59)=0,"",SUMPRODUCT((Items!$B$5:$B$59=A10)*Items!$G$5:$G$59)/SUMPRODUCT((Items!$B$5:$B$59=A10)*Items!$H$5:$H$59))</f>
         <v/>
       </c>
     </row>
@@ -8390,11 +8789,11 @@
         </is>
       </c>
       <c r="C11">
-        <f>COUNTIF(Items!$B$5:$B$56,A11)</f>
+        <f>COUNTIF(Items!$B$5:$B$59,A11)</f>
         <v/>
       </c>
       <c r="D11" s="6">
-        <f>IF(SUMPRODUCT((Items!$B$5:$B$56=A11)*Items!$H$5:$H$56)=0,"",SUMPRODUCT((Items!$B$5:$B$56=A11)*Items!$G$5:$G$56)/SUMPRODUCT((Items!$B$5:$B$56=A11)*Items!$H$5:$H$56))</f>
+        <f>IF(SUMPRODUCT((Items!$B$5:$B$59=A11)*Items!$H$5:$H$59)=0,"",SUMPRODUCT((Items!$B$5:$B$59=A11)*Items!$G$5:$G$59)/SUMPRODUCT((Items!$B$5:$B$59=A11)*Items!$H$5:$H$59))</f>
         <v/>
       </c>
     </row>
@@ -8408,11 +8807,11 @@
         </is>
       </c>
       <c r="C12">
-        <f>COUNTIF(Items!$B$5:$B$56,A12)</f>
+        <f>COUNTIF(Items!$B$5:$B$59,A12)</f>
         <v/>
       </c>
       <c r="D12" s="6">
-        <f>IF(SUMPRODUCT((Items!$B$5:$B$56=A12)*Items!$H$5:$H$56)=0,"",SUMPRODUCT((Items!$B$5:$B$56=A12)*Items!$G$5:$G$56)/SUMPRODUCT((Items!$B$5:$B$56=A12)*Items!$H$5:$H$56))</f>
+        <f>IF(SUMPRODUCT((Items!$B$5:$B$59=A12)*Items!$H$5:$H$59)=0,"",SUMPRODUCT((Items!$B$5:$B$59=A12)*Items!$G$5:$G$59)/SUMPRODUCT((Items!$B$5:$B$59=A12)*Items!$H$5:$H$59))</f>
         <v/>
       </c>
     </row>
@@ -8426,11 +8825,11 @@
         </is>
       </c>
       <c r="C13">
-        <f>COUNTIF(Items!$B$5:$B$56,A13)</f>
+        <f>COUNTIF(Items!$B$5:$B$59,A13)</f>
         <v/>
       </c>
       <c r="D13" s="6">
-        <f>IF(SUMPRODUCT((Items!$B$5:$B$56=A13)*Items!$H$5:$H$56)=0,"",SUMPRODUCT((Items!$B$5:$B$56=A13)*Items!$G$5:$G$56)/SUMPRODUCT((Items!$B$5:$B$56=A13)*Items!$H$5:$H$56))</f>
+        <f>IF(SUMPRODUCT((Items!$B$5:$B$59=A13)*Items!$H$5:$H$59)=0,"",SUMPRODUCT((Items!$B$5:$B$59=A13)*Items!$G$5:$G$59)/SUMPRODUCT((Items!$B$5:$B$59=A13)*Items!$H$5:$H$59))</f>
         <v/>
       </c>
     </row>
@@ -8482,15 +8881,15 @@
         <v>1</v>
       </c>
       <c r="B5" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$5:$BA$5))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$5:$BA$5=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$5:$BA$5)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$5:$BD$5))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$5:$BD$5=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$5:$BD$5)))</f>
         <v/>
       </c>
       <c r="C5" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$5:$BA$5))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$5:$BA$5=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$5:$BA$5)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$5:$BD$5))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$5:$BD$5=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$5:$BD$5)))</f>
         <v/>
       </c>
       <c r="D5" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$5:$BA$5))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$5:$BA$5=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$5:$BA$5)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$5:$BD$5))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$5:$BD$5=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$5:$BD$5)))</f>
         <v/>
       </c>
     </row>
@@ -8499,15 +8898,15 @@
         <v>2</v>
       </c>
       <c r="B6" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$6:$BA$6))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$6:$BA$6=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$6:$BA$6)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$6:$BD$6))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$6:$BD$6=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$6:$BD$6)))</f>
         <v/>
       </c>
       <c r="C6" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$6:$BA$6))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$6:$BA$6=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$6:$BA$6)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$6:$BD$6))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$6:$BD$6=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$6:$BD$6)))</f>
         <v/>
       </c>
       <c r="D6" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$6:$BA$6))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$6:$BA$6=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$6:$BA$6)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$6:$BD$6))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$6:$BD$6=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$6:$BD$6)))</f>
         <v/>
       </c>
     </row>
@@ -8516,15 +8915,15 @@
         <v>3</v>
       </c>
       <c r="B7" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$7:$BA$7))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$7:$BA$7=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$7:$BA$7)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$7:$BD$7))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$7:$BD$7=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$7:$BD$7)))</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$7:$BA$7))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$7:$BA$7=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$7:$BA$7)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$7:$BD$7))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$7:$BD$7=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$7:$BD$7)))</f>
         <v/>
       </c>
       <c r="D7" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$7:$BA$7))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$7:$BA$7=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$7:$BA$7)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$7:$BD$7))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$7:$BD$7=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$7:$BD$7)))</f>
         <v/>
       </c>
     </row>
@@ -8533,15 +8932,15 @@
         <v>4</v>
       </c>
       <c r="B8" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$8:$BA$8))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$8:$BA$8=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$8:$BA$8)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$8:$BD$8))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$8:$BD$8=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$8:$BD$8)))</f>
         <v/>
       </c>
       <c r="C8" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$8:$BA$8))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$8:$BA$8=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$8:$BA$8)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$8:$BD$8))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$8:$BD$8=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$8:$BD$8)))</f>
         <v/>
       </c>
       <c r="D8" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$8:$BA$8))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$8:$BA$8=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$8:$BA$8)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$8:$BD$8))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$8:$BD$8=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$8:$BD$8)))</f>
         <v/>
       </c>
     </row>
@@ -8550,15 +8949,15 @@
         <v>5</v>
       </c>
       <c r="B9" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$9:$BA$9))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$9:$BA$9=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$9:$BA$9)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$9:$BD$9))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$9:$BD$9=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$9:$BD$9)))</f>
         <v/>
       </c>
       <c r="C9" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$9:$BA$9))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$9:$BA$9=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$9:$BA$9)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$9:$BD$9))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$9:$BD$9=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$9:$BD$9)))</f>
         <v/>
       </c>
       <c r="D9" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$9:$BA$9))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$9:$BA$9=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$9:$BA$9)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$9:$BD$9))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$9:$BD$9=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$9:$BD$9)))</f>
         <v/>
       </c>
     </row>
@@ -8567,15 +8966,15 @@
         <v>6</v>
       </c>
       <c r="B10" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$10:$BA$10))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$10:$BA$10=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$10:$BA$10)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$10:$BD$10))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$10:$BD$10=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$10:$BD$10)))</f>
         <v/>
       </c>
       <c r="C10" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$10:$BA$10))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$10:$BA$10=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$10:$BA$10)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$10:$BD$10))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$10:$BD$10=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$10:$BD$10)))</f>
         <v/>
       </c>
       <c r="D10" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$10:$BA$10))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$10:$BA$10=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$10:$BA$10)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$10:$BD$10))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$10:$BD$10=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$10:$BD$10)))</f>
         <v/>
       </c>
     </row>
@@ -8584,15 +8983,15 @@
         <v>7</v>
       </c>
       <c r="B11" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$11:$BA$11))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$11:$BA$11=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$11:$BA$11)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$11:$BD$11))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$11:$BD$11=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$11:$BD$11)))</f>
         <v/>
       </c>
       <c r="C11" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$11:$BA$11))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$11:$BA$11=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$11:$BA$11)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$11:$BD$11))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$11:$BD$11=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$11:$BD$11)))</f>
         <v/>
       </c>
       <c r="D11" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$11:$BA$11))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$11:$BA$11=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$11:$BA$11)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$11:$BD$11))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$11:$BD$11=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$11:$BD$11)))</f>
         <v/>
       </c>
     </row>
@@ -8601,15 +9000,15 @@
         <v>8</v>
       </c>
       <c r="B12" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$12:$BA$12))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$12:$BA$12=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$12:$BA$12)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$12:$BD$12))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$12:$BD$12=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$12:$BD$12)))</f>
         <v/>
       </c>
       <c r="C12" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$12:$BA$12))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$12:$BA$12=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$12:$BA$12)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$12:$BD$12))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$12:$BD$12=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$12:$BD$12)))</f>
         <v/>
       </c>
       <c r="D12" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$12:$BA$12))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$12:$BA$12=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$12:$BA$12)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$12:$BD$12))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$12:$BD$12=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$12:$BD$12)))</f>
         <v/>
       </c>
     </row>
@@ -8618,15 +9017,15 @@
         <v>9</v>
       </c>
       <c r="B13" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$13:$BA$13))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$13:$BA$13=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$13:$BA$13)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$13:$BD$13))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$13:$BD$13=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$13:$BD$13)))</f>
         <v/>
       </c>
       <c r="C13" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$13:$BA$13))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$13:$BA$13=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$13:$BA$13)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$13:$BD$13))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$13:$BD$13=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$13:$BD$13)))</f>
         <v/>
       </c>
       <c r="D13" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$13:$BA$13))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$13:$BA$13=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$13:$BA$13)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$13:$BD$13))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$13:$BD$13=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$13:$BD$13)))</f>
         <v/>
       </c>
     </row>
@@ -8635,15 +9034,15 @@
         <v>10</v>
       </c>
       <c r="B14" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$14:$BA$14))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$14:$BA$14=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$14:$BA$14)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$14:$BD$14))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$14:$BD$14=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$14:$BD$14)))</f>
         <v/>
       </c>
       <c r="C14" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$14:$BA$14))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$14:$BA$14=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$14:$BA$14)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$14:$BD$14))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$14:$BD$14=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$14:$BD$14)))</f>
         <v/>
       </c>
       <c r="D14" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$14:$BA$14))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$14:$BA$14=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$14:$BA$14)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$14:$BD$14))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$14:$BD$14=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$14:$BD$14)))</f>
         <v/>
       </c>
     </row>
@@ -8652,15 +9051,15 @@
         <v>11</v>
       </c>
       <c r="B15" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$15:$BA$15))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$15:$BA$15=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$15:$BA$15)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$15:$BD$15))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$15:$BD$15=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$15:$BD$15)))</f>
         <v/>
       </c>
       <c r="C15" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$15:$BA$15))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$15:$BA$15=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$15:$BA$15)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$15:$BD$15))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$15:$BD$15=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$15:$BD$15)))</f>
         <v/>
       </c>
       <c r="D15" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$15:$BA$15))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$15:$BA$15=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$15:$BA$15)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$15:$BD$15))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$15:$BD$15=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$15:$BD$15)))</f>
         <v/>
       </c>
     </row>
@@ -8669,15 +9068,15 @@
         <v>12</v>
       </c>
       <c r="B16" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$16:$BA$16))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$16:$BA$16=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$16:$BA$16)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$16:$BD$16))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$16:$BD$16=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$16:$BD$16)))</f>
         <v/>
       </c>
       <c r="C16" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$16:$BA$16))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$16:$BA$16=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$16:$BA$16)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$16:$BD$16))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$16:$BD$16=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$16:$BD$16)))</f>
         <v/>
       </c>
       <c r="D16" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$16:$BA$16))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$16:$BA$16=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$16:$BA$16)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$16:$BD$16))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$16:$BD$16=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$16:$BD$16)))</f>
         <v/>
       </c>
     </row>
@@ -8686,15 +9085,15 @@
         <v>13</v>
       </c>
       <c r="B17" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$17:$BA$17))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$17:$BA$17=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$17:$BA$17)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$17:$BD$17))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$17:$BD$17=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$17:$BD$17)))</f>
         <v/>
       </c>
       <c r="C17" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$17:$BA$17))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$17:$BA$17=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$17:$BA$17)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$17:$BD$17))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$17:$BD$17=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$17:$BD$17)))</f>
         <v/>
       </c>
       <c r="D17" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$17:$BA$17))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$17:$BA$17=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$17:$BA$17)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$17:$BD$17))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$17:$BD$17=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$17:$BD$17)))</f>
         <v/>
       </c>
     </row>
@@ -8703,15 +9102,15 @@
         <v>14</v>
       </c>
       <c r="B18" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$18:$BA$18))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$18:$BA$18=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$18:$BA$18)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$18:$BD$18))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$18:$BD$18=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$18:$BD$18)))</f>
         <v/>
       </c>
       <c r="C18" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$18:$BA$18))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$18:$BA$18=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$18:$BA$18)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$18:$BD$18))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$18:$BD$18=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$18:$BD$18)))</f>
         <v/>
       </c>
       <c r="D18" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$18:$BA$18))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$18:$BA$18=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$18:$BA$18)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$18:$BD$18))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$18:$BD$18=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$18:$BD$18)))</f>
         <v/>
       </c>
     </row>
@@ -8720,15 +9119,15 @@
         <v>15</v>
       </c>
       <c r="B19" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$19:$BA$19))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$19:$BA$19=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$19:$BA$19)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$19:$BD$19))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$19:$BD$19=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$19:$BD$19)))</f>
         <v/>
       </c>
       <c r="C19" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$19:$BA$19))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$19:$BA$19=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$19:$BA$19)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$19:$BD$19))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$19:$BD$19=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$19:$BD$19)))</f>
         <v/>
       </c>
       <c r="D19" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$19:$BA$19))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$19:$BA$19=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$19:$BA$19)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$19:$BD$19))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$19:$BD$19=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$19:$BD$19)))</f>
         <v/>
       </c>
     </row>
@@ -8737,15 +9136,15 @@
         <v>16</v>
       </c>
       <c r="B20" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$20:$BA$20))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$20:$BA$20=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$20:$BA$20)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$20:$BD$20))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$20:$BD$20=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$20:$BD$20)))</f>
         <v/>
       </c>
       <c r="C20" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$20:$BA$20))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$20:$BA$20=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$20:$BA$20)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$20:$BD$20))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$20:$BD$20=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$20:$BD$20)))</f>
         <v/>
       </c>
       <c r="D20" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$20:$BA$20))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$20:$BA$20=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$20:$BA$20)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$20:$BD$20))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$20:$BD$20=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$20:$BD$20)))</f>
         <v/>
       </c>
     </row>
@@ -8754,15 +9153,15 @@
         <v>17</v>
       </c>
       <c r="B21" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$21:$BA$21))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$21:$BA$21=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$21:$BA$21)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$21:$BD$21))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$21:$BD$21=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$21:$BD$21)))</f>
         <v/>
       </c>
       <c r="C21" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$21:$BA$21))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$21:$BA$21=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$21:$BA$21)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$21:$BD$21))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$21:$BD$21=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$21:$BD$21)))</f>
         <v/>
       </c>
       <c r="D21" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$21:$BA$21))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$21:$BA$21=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$21:$BA$21)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$21:$BD$21))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$21:$BD$21=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$21:$BD$21)))</f>
         <v/>
       </c>
     </row>
@@ -8771,15 +9170,15 @@
         <v>18</v>
       </c>
       <c r="B22" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$22:$BA$22))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$22:$BA$22=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$22:$BA$22)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$22:$BD$22))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$22:$BD$22=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$22:$BD$22)))</f>
         <v/>
       </c>
       <c r="C22" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$22:$BA$22))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$22:$BA$22=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$22:$BA$22)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$22:$BD$22))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$22:$BD$22=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$22:$BD$22)))</f>
         <v/>
       </c>
       <c r="D22" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$22:$BA$22))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$22:$BA$22=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$22:$BA$22)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$22:$BD$22))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$22:$BD$22=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$22:$BD$22)))</f>
         <v/>
       </c>
     </row>
@@ -8788,15 +9187,15 @@
         <v>19</v>
       </c>
       <c r="B23" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$23:$BA$23))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$23:$BA$23=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$23:$BA$23)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$23:$BD$23))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$23:$BD$23=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$23:$BD$23)))</f>
         <v/>
       </c>
       <c r="C23" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$23:$BA$23))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$23:$BA$23=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$23:$BA$23)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$23:$BD$23))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$23:$BD$23=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$23:$BD$23)))</f>
         <v/>
       </c>
       <c r="D23" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$23:$BA$23))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$23:$BA$23=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$23:$BA$23)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$23:$BD$23))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$23:$BD$23=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$23:$BD$23)))</f>
         <v/>
       </c>
     </row>
@@ -8805,15 +9204,15 @@
         <v>20</v>
       </c>
       <c r="B24" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$24:$BA$24))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$24:$BA$24=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$24:$BA$24)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$24:$BD$24))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$24:$BD$24=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$24:$BD$24)))</f>
         <v/>
       </c>
       <c r="C24" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$24:$BA$24))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$24:$BA$24=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$24:$BA$24)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$24:$BD$24))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$24:$BD$24=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$24:$BD$24)))</f>
         <v/>
       </c>
       <c r="D24" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$24:$BA$24))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$24:$BA$24=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$24:$BA$24)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$24:$BD$24))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$24:$BD$24=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$24:$BD$24)))</f>
         <v/>
       </c>
     </row>
@@ -8822,15 +9221,15 @@
         <v>21</v>
       </c>
       <c r="B25" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$25:$BA$25))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$25:$BA$25=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$25:$BA$25)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$25:$BD$25))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$25:$BD$25=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$25:$BD$25)))</f>
         <v/>
       </c>
       <c r="C25" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$25:$BA$25))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$25:$BA$25=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$25:$BA$25)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$25:$BD$25))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$25:$BD$25=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$25:$BD$25)))</f>
         <v/>
       </c>
       <c r="D25" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$25:$BA$25))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$25:$BA$25=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$25:$BA$25)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$25:$BD$25))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$25:$BD$25=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$25:$BD$25)))</f>
         <v/>
       </c>
     </row>
@@ -8839,15 +9238,15 @@
         <v>22</v>
       </c>
       <c r="B26" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$26:$BA$26))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$26:$BA$26=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$26:$BA$26)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$26:$BD$26))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$26:$BD$26=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$26:$BD$26)))</f>
         <v/>
       </c>
       <c r="C26" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$26:$BA$26))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$26:$BA$26=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$26:$BA$26)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$26:$BD$26))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$26:$BD$26=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$26:$BD$26)))</f>
         <v/>
       </c>
       <c r="D26" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$26:$BA$26))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$26:$BA$26=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$26:$BA$26)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$26:$BD$26))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$26:$BD$26=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$26:$BD$26)))</f>
         <v/>
       </c>
     </row>
@@ -8856,15 +9255,15 @@
         <v>23</v>
       </c>
       <c r="B27" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$27:$BA$27))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$27:$BA$27=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$27:$BA$27)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$27:$BD$27))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$27:$BD$27=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$27:$BD$27)))</f>
         <v/>
       </c>
       <c r="C27" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$27:$BA$27))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$27:$BA$27=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$27:$BA$27)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$27:$BD$27))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$27:$BD$27=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$27:$BD$27)))</f>
         <v/>
       </c>
       <c r="D27" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$27:$BA$27))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$27:$BA$27=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$27:$BA$27)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$27:$BD$27))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$27:$BD$27=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$27:$BD$27)))</f>
         <v/>
       </c>
     </row>
@@ -8873,15 +9272,15 @@
         <v>24</v>
       </c>
       <c r="B28" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$28:$BA$28))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$28:$BA$28=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$28:$BA$28)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$28:$BD$28))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$28:$BD$28=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$28:$BD$28)))</f>
         <v/>
       </c>
       <c r="C28" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$28:$BA$28))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$28:$BA$28=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$28:$BA$28)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$28:$BD$28))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$28:$BD$28=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$28:$BD$28)))</f>
         <v/>
       </c>
       <c r="D28" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$28:$BA$28))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$28:$BA$28=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$28:$BA$28)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$28:$BD$28))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$28:$BD$28=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$28:$BD$28)))</f>
         <v/>
       </c>
     </row>
@@ -8890,15 +9289,15 @@
         <v>25</v>
       </c>
       <c r="B29" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$29:$BA$29))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$29:$BA$29=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$29:$BA$29)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$29:$BD$29))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$29:$BD$29=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$29:$BD$29)))</f>
         <v/>
       </c>
       <c r="C29" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$29:$BA$29))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$29:$BA$29=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$29:$BA$29)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$29:$BD$29))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$29:$BD$29=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$29:$BD$29)))</f>
         <v/>
       </c>
       <c r="D29" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$29:$BA$29))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$29:$BA$29=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$29:$BA$29)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$29:$BD$29))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$29:$BD$29=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$29:$BD$29)))</f>
         <v/>
       </c>
     </row>
@@ -8907,15 +9306,15 @@
         <v>26</v>
       </c>
       <c r="B30" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$30:$BA$30))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$30:$BA$30=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$30:$BA$30)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$30:$BD$30))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$30:$BD$30=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$30:$BD$30)))</f>
         <v/>
       </c>
       <c r="C30" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$30:$BA$30))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$30:$BA$30=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$30:$BA$30)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$30:$BD$30))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$30:$BD$30=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$30:$BD$30)))</f>
         <v/>
       </c>
       <c r="D30" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$30:$BA$30))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$30:$BA$30=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$30:$BA$30)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$30:$BD$30))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$30:$BD$30=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$30:$BD$30)))</f>
         <v/>
       </c>
     </row>
@@ -8924,15 +9323,15 @@
         <v>27</v>
       </c>
       <c r="B31" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$31:$BA$31))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$31:$BA$31=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$31:$BA$31)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$31:$BD$31))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$31:$BD$31=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$31:$BD$31)))</f>
         <v/>
       </c>
       <c r="C31" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$31:$BA$31))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$31:$BA$31=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$31:$BA$31)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$31:$BD$31))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$31:$BD$31=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$31:$BD$31)))</f>
         <v/>
       </c>
       <c r="D31" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$31:$BA$31))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$31:$BA$31=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$31:$BA$31)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$31:$BD$31))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$31:$BD$31=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$31:$BD$31)))</f>
         <v/>
       </c>
     </row>
@@ -8941,15 +9340,15 @@
         <v>28</v>
       </c>
       <c r="B32" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$32:$BA$32))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$32:$BA$32=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$32:$BA$32)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$32:$BD$32))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$32:$BD$32=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$32:$BD$32)))</f>
         <v/>
       </c>
       <c r="C32" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$32:$BA$32))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$32:$BA$32=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$32:$BA$32)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$32:$BD$32))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$32:$BD$32=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$32:$BD$32)))</f>
         <v/>
       </c>
       <c r="D32" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$32:$BA$32))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$32:$BA$32=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$32:$BA$32)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$32:$BD$32))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$32:$BD$32=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$32:$BD$32)))</f>
         <v/>
       </c>
     </row>
@@ -8958,15 +9357,15 @@
         <v>29</v>
       </c>
       <c r="B33" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$33:$BA$33))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$33:$BA$33=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$33:$BA$33)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$33:$BD$33))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$33:$BD$33=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$33:$BD$33)))</f>
         <v/>
       </c>
       <c r="C33" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$33:$BA$33))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$33:$BA$33=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$33:$BA$33)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$33:$BD$33))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$33:$BD$33=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$33:$BD$33)))</f>
         <v/>
       </c>
       <c r="D33" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$33:$BA$33))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$33:$BA$33=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$33:$BA$33)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$33:$BD$33))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$33:$BD$33=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$33:$BD$33)))</f>
         <v/>
       </c>
     </row>
@@ -8975,15 +9374,15 @@
         <v>30</v>
       </c>
       <c r="B34" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$34:$BA$34))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$34:$BA$34=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$34:$BA$34)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$34:$BD$34))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$34:$BD$34=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$34:$BD$34)))</f>
         <v/>
       </c>
       <c r="C34" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$34:$BA$34))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$34:$BA$34=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$34:$BA$34)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$34:$BD$34))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$34:$BD$34=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$34:$BD$34)))</f>
         <v/>
       </c>
       <c r="D34" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$34:$BA$34))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$34:$BA$34=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$34:$BA$34)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$34:$BD$34))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$34:$BD$34=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$34:$BD$34)))</f>
         <v/>
       </c>
     </row>
@@ -8992,15 +9391,15 @@
         <v>31</v>
       </c>
       <c r="B35" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$35:$BA$35))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$35:$BA$35=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$35:$BA$35)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$35:$BD$35))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$35:$BD$35=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$35:$BD$35)))</f>
         <v/>
       </c>
       <c r="C35" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$35:$BA$35))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$35:$BA$35=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$35:$BA$35)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$35:$BD$35))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$35:$BD$35=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$35:$BD$35)))</f>
         <v/>
       </c>
       <c r="D35" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$35:$BA$35))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$35:$BA$35=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$35:$BA$35)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$35:$BD$35))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$35:$BD$35=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$35:$BD$35)))</f>
         <v/>
       </c>
     </row>
@@ -9009,15 +9408,15 @@
         <v>32</v>
       </c>
       <c r="B36" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$36:$BA$36))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$36:$BA$36=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$36:$BA$36)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$36:$BD$36))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$36:$BD$36=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$36:$BD$36)))</f>
         <v/>
       </c>
       <c r="C36" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$36:$BA$36))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$36:$BA$36=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$36:$BA$36)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$36:$BD$36))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$36:$BD$36=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$36:$BD$36)))</f>
         <v/>
       </c>
       <c r="D36" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$36:$BA$36))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$36:$BA$36=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$36:$BA$36)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$36:$BD$36))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$36:$BD$36=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$36:$BD$36)))</f>
         <v/>
       </c>
     </row>
@@ -9026,15 +9425,15 @@
         <v>33</v>
       </c>
       <c r="B37" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$37:$BA$37))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$37:$BA$37=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$37:$BA$37)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$37:$BD$37))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$37:$BD$37=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$37:$BD$37)))</f>
         <v/>
       </c>
       <c r="C37" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$37:$BA$37))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$37:$BA$37=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$37:$BA$37)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$37:$BD$37))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$37:$BD$37=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$37:$BD$37)))</f>
         <v/>
       </c>
       <c r="D37" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$37:$BA$37))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$37:$BA$37=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$37:$BA$37)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$37:$BD$37))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$37:$BD$37=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$37:$BD$37)))</f>
         <v/>
       </c>
     </row>
@@ -9043,15 +9442,15 @@
         <v>34</v>
       </c>
       <c r="B38" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$38:$BA$38))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$38:$BA$38=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$38:$BA$38)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$38:$BD$38))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$38:$BD$38=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$38:$BD$38)))</f>
         <v/>
       </c>
       <c r="C38" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$38:$BA$38))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$38:$BA$38=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$38:$BA$38)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$38:$BD$38))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$38:$BD$38=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$38:$BD$38)))</f>
         <v/>
       </c>
       <c r="D38" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$38:$BA$38))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$38:$BA$38=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$38:$BA$38)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$38:$BD$38))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$38:$BD$38=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$38:$BD$38)))</f>
         <v/>
       </c>
     </row>
@@ -9060,15 +9459,15 @@
         <v>35</v>
       </c>
       <c r="B39" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$39:$BA$39))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*(Marks!$B$39:$BA$39=1))/SUMPRODUCT((Marks!$B$3:$BA$3=B$4)*ISNUMBER(Marks!$B$39:$BA$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$39:$BD$39))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*(Marks!$B$39:$BD$39=1))/SUMPRODUCT((Marks!$B$3:$BD$3=B$4)*ISNUMBER(Marks!$B$39:$BD$39)))</f>
         <v/>
       </c>
       <c r="C39" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$39:$BA$39))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*(Marks!$B$39:$BA$39=1))/SUMPRODUCT((Marks!$B$3:$BA$3=C$4)*ISNUMBER(Marks!$B$39:$BA$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$39:$BD$39))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*(Marks!$B$39:$BD$39=1))/SUMPRODUCT((Marks!$B$3:$BD$3=C$4)*ISNUMBER(Marks!$B$39:$BD$39)))</f>
         <v/>
       </c>
       <c r="D39" s="6">
-        <f>IF(SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$39:$BA$39))=0,"",SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*(Marks!$B$39:$BA$39=1))/SUMPRODUCT((Marks!$B$3:$BA$3=D$4)*ISNUMBER(Marks!$B$39:$BA$39)))</f>
+        <f>IF(SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$39:$BD$39))=0,"",SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*(Marks!$B$39:$BD$39=1))/SUMPRODUCT((Marks!$B$3:$BD$3=D$4)*ISNUMBER(Marks!$B$39:$BD$39)))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
W02 Saturday paper and key rebuilt in the diagnostic's Word format
Built with build_saturday_paper.py W02 --docx on the merged builder: the Word
paper opens on the purpose, the rules with the Company row, step one's ratings,
the paper at a glance and the pacing ribbon, prints every item with its label,
and closes on a one-page answer sheet; the key ends on the marking grid, and
the workbook gains its Ratings sheet, which xlsx_recalc.py passes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P7zaoR4dQ5pzBFnsX549JQ
</commit_message>
<xml_diff>
--- a/content/W02/SAT/answer-key/C2_W02_SAT_item_analysis_TRAINER.xlsx
+++ b/content/W02/SAT/answer-key/C2_W02_SAT_item_analysis_TRAINER.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Discussion" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tags" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Seats" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ratings" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +22,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="4">
     <font>
       <name val="Calibri"/>
@@ -69,7 +72,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -81,6 +84,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -9474,4 +9478,1508 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N48"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="44" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Step one: each part's rating beside its score</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Type each seat's ratings, 1 to 4, from the answer sheet; the rates on the right are computed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K3" t="n">
+        <v>3</v>
+      </c>
+      <c r="L3" t="n">
+        <v>4</v>
+      </c>
+      <c r="M3" t="n">
+        <v>5</v>
+      </c>
+      <c r="N3" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Seat</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Rating, part 1</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Rating, part 2</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Rating, part 3</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Rating, part 4</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Rating, part 5</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Rating, part 6</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>Right rate, part 1</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Right rate, part 2</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Right rate, part 3</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Right rate, part 4</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>Right rate, part 5</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>Right rate, part 6</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n"/>
+      <c r="E5" s="5" t="n"/>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+      <c r="I5" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$5:$BD$5))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$5:$BD$5=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$5:$BD$5)))</f>
+        <v/>
+      </c>
+      <c r="J5" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$5:$BD$5))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$5:$BD$5=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$5:$BD$5)))</f>
+        <v/>
+      </c>
+      <c r="K5" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$5:$BD$5))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$5:$BD$5=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$5:$BD$5)))</f>
+        <v/>
+      </c>
+      <c r="L5" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$5:$BD$5))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$5:$BD$5=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$5:$BD$5)))</f>
+        <v/>
+      </c>
+      <c r="M5" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$5:$BD$5))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$5:$BD$5=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$5:$BD$5)))</f>
+        <v/>
+      </c>
+      <c r="N5" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$5:$BD$5))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$5:$BD$5=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$5:$BD$5)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="I6" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$6:$BD$6))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$6:$BD$6=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$6:$BD$6)))</f>
+        <v/>
+      </c>
+      <c r="J6" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$6:$BD$6))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$6:$BD$6=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$6:$BD$6)))</f>
+        <v/>
+      </c>
+      <c r="K6" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$6:$BD$6))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$6:$BD$6=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$6:$BD$6)))</f>
+        <v/>
+      </c>
+      <c r="L6" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$6:$BD$6))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$6:$BD$6=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$6:$BD$6)))</f>
+        <v/>
+      </c>
+      <c r="M6" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$6:$BD$6))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$6:$BD$6=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$6:$BD$6)))</f>
+        <v/>
+      </c>
+      <c r="N6" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$6:$BD$6))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$6:$BD$6=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$6:$BD$6)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="5" t="n"/>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
+      <c r="F7" s="5" t="n"/>
+      <c r="G7" s="5" t="n"/>
+      <c r="I7" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$7:$BD$7))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$7:$BD$7=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$7:$BD$7)))</f>
+        <v/>
+      </c>
+      <c r="J7" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$7:$BD$7))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$7:$BD$7=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$7:$BD$7)))</f>
+        <v/>
+      </c>
+      <c r="K7" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$7:$BD$7))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$7:$BD$7=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$7:$BD$7)))</f>
+        <v/>
+      </c>
+      <c r="L7" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$7:$BD$7))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$7:$BD$7=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$7:$BD$7)))</f>
+        <v/>
+      </c>
+      <c r="M7" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$7:$BD$7))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$7:$BD$7=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$7:$BD$7)))</f>
+        <v/>
+      </c>
+      <c r="N7" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$7:$BD$7))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$7:$BD$7=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$7:$BD$7)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="5" t="n"/>
+      <c r="D8" s="5" t="n"/>
+      <c r="E8" s="5" t="n"/>
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="5" t="n"/>
+      <c r="I8" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$8:$BD$8))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$8:$BD$8=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$8:$BD$8)))</f>
+        <v/>
+      </c>
+      <c r="J8" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$8:$BD$8))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$8:$BD$8=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$8:$BD$8)))</f>
+        <v/>
+      </c>
+      <c r="K8" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$8:$BD$8))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$8:$BD$8=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$8:$BD$8)))</f>
+        <v/>
+      </c>
+      <c r="L8" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$8:$BD$8))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$8:$BD$8=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$8:$BD$8)))</f>
+        <v/>
+      </c>
+      <c r="M8" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$8:$BD$8))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$8:$BD$8=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$8:$BD$8)))</f>
+        <v/>
+      </c>
+      <c r="N8" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$8:$BD$8))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$8:$BD$8=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$8:$BD$8)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="I9" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$9:$BD$9))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$9:$BD$9=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$9:$BD$9)))</f>
+        <v/>
+      </c>
+      <c r="J9" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$9:$BD$9))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$9:$BD$9=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$9:$BD$9)))</f>
+        <v/>
+      </c>
+      <c r="K9" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$9:$BD$9))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$9:$BD$9=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$9:$BD$9)))</f>
+        <v/>
+      </c>
+      <c r="L9" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$9:$BD$9))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$9:$BD$9=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$9:$BD$9)))</f>
+        <v/>
+      </c>
+      <c r="M9" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$9:$BD$9))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$9:$BD$9=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$9:$BD$9)))</f>
+        <v/>
+      </c>
+      <c r="N9" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$9:$BD$9))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$9:$BD$9=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$9:$BD$9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="5" t="n"/>
+      <c r="F10" s="5" t="n"/>
+      <c r="G10" s="5" t="n"/>
+      <c r="I10" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$10:$BD$10))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$10:$BD$10=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$10:$BD$10)))</f>
+        <v/>
+      </c>
+      <c r="J10" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$10:$BD$10))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$10:$BD$10=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$10:$BD$10)))</f>
+        <v/>
+      </c>
+      <c r="K10" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$10:$BD$10))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$10:$BD$10=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$10:$BD$10)))</f>
+        <v/>
+      </c>
+      <c r="L10" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$10:$BD$10))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$10:$BD$10=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$10:$BD$10)))</f>
+        <v/>
+      </c>
+      <c r="M10" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$10:$BD$10))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$10:$BD$10=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$10:$BD$10)))</f>
+        <v/>
+      </c>
+      <c r="N10" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$10:$BD$10))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$10:$BD$10=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$10:$BD$10)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
+      <c r="I11" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$11:$BD$11))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$11:$BD$11=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$11:$BD$11)))</f>
+        <v/>
+      </c>
+      <c r="J11" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$11:$BD$11))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$11:$BD$11=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$11:$BD$11)))</f>
+        <v/>
+      </c>
+      <c r="K11" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$11:$BD$11))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$11:$BD$11=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$11:$BD$11)))</f>
+        <v/>
+      </c>
+      <c r="L11" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$11:$BD$11))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$11:$BD$11=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$11:$BD$11)))</f>
+        <v/>
+      </c>
+      <c r="M11" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$11:$BD$11))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$11:$BD$11=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$11:$BD$11)))</f>
+        <v/>
+      </c>
+      <c r="N11" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$11:$BD$11))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$11:$BD$11=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$11:$BD$11)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="5" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="5" t="n"/>
+      <c r="F12" s="5" t="n"/>
+      <c r="G12" s="5" t="n"/>
+      <c r="I12" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$12:$BD$12))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$12:$BD$12=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$12:$BD$12)))</f>
+        <v/>
+      </c>
+      <c r="J12" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$12:$BD$12))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$12:$BD$12=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$12:$BD$12)))</f>
+        <v/>
+      </c>
+      <c r="K12" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$12:$BD$12))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$12:$BD$12=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$12:$BD$12)))</f>
+        <v/>
+      </c>
+      <c r="L12" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$12:$BD$12))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$12:$BD$12=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$12:$BD$12)))</f>
+        <v/>
+      </c>
+      <c r="M12" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$12:$BD$12))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$12:$BD$12=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$12:$BD$12)))</f>
+        <v/>
+      </c>
+      <c r="N12" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$12:$BD$12))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$12:$BD$12=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$12:$BD$12)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="5" t="n"/>
+      <c r="C13" s="5" t="n"/>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="n"/>
+      <c r="I13" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$13:$BD$13))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$13:$BD$13=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$13:$BD$13)))</f>
+        <v/>
+      </c>
+      <c r="J13" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$13:$BD$13))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$13:$BD$13=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$13:$BD$13)))</f>
+        <v/>
+      </c>
+      <c r="K13" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$13:$BD$13))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$13:$BD$13=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$13:$BD$13)))</f>
+        <v/>
+      </c>
+      <c r="L13" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$13:$BD$13))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$13:$BD$13=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$13:$BD$13)))</f>
+        <v/>
+      </c>
+      <c r="M13" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$13:$BD$13))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$13:$BD$13=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$13:$BD$13)))</f>
+        <v/>
+      </c>
+      <c r="N13" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$13:$BD$13))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$13:$BD$13=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$13:$BD$13)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="5" t="n"/>
+      <c r="C14" s="5" t="n"/>
+      <c r="D14" s="5" t="n"/>
+      <c r="E14" s="5" t="n"/>
+      <c r="F14" s="5" t="n"/>
+      <c r="G14" s="5" t="n"/>
+      <c r="I14" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$14:$BD$14))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$14:$BD$14=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$14:$BD$14)))</f>
+        <v/>
+      </c>
+      <c r="J14" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$14:$BD$14))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$14:$BD$14=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$14:$BD$14)))</f>
+        <v/>
+      </c>
+      <c r="K14" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$14:$BD$14))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$14:$BD$14=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$14:$BD$14)))</f>
+        <v/>
+      </c>
+      <c r="L14" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$14:$BD$14))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$14:$BD$14=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$14:$BD$14)))</f>
+        <v/>
+      </c>
+      <c r="M14" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$14:$BD$14))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$14:$BD$14=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$14:$BD$14)))</f>
+        <v/>
+      </c>
+      <c r="N14" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$14:$BD$14))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$14:$BD$14=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$14:$BD$14)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="5" t="n"/>
+      <c r="C15" s="5" t="n"/>
+      <c r="D15" s="5" t="n"/>
+      <c r="E15" s="5" t="n"/>
+      <c r="F15" s="5" t="n"/>
+      <c r="G15" s="5" t="n"/>
+      <c r="I15" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$15:$BD$15))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$15:$BD$15=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$15:$BD$15)))</f>
+        <v/>
+      </c>
+      <c r="J15" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$15:$BD$15))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$15:$BD$15=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$15:$BD$15)))</f>
+        <v/>
+      </c>
+      <c r="K15" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$15:$BD$15))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$15:$BD$15=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$15:$BD$15)))</f>
+        <v/>
+      </c>
+      <c r="L15" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$15:$BD$15))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$15:$BD$15=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$15:$BD$15)))</f>
+        <v/>
+      </c>
+      <c r="M15" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$15:$BD$15))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$15:$BD$15=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$15:$BD$15)))</f>
+        <v/>
+      </c>
+      <c r="N15" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$15:$BD$15))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$15:$BD$15=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$15:$BD$15)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="5" t="n"/>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="5" t="n"/>
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="5" t="n"/>
+      <c r="G16" s="5" t="n"/>
+      <c r="I16" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$16:$BD$16))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$16:$BD$16=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$16:$BD$16)))</f>
+        <v/>
+      </c>
+      <c r="J16" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$16:$BD$16))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$16:$BD$16=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$16:$BD$16)))</f>
+        <v/>
+      </c>
+      <c r="K16" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$16:$BD$16))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$16:$BD$16=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$16:$BD$16)))</f>
+        <v/>
+      </c>
+      <c r="L16" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$16:$BD$16))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$16:$BD$16=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$16:$BD$16)))</f>
+        <v/>
+      </c>
+      <c r="M16" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$16:$BD$16))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$16:$BD$16=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$16:$BD$16)))</f>
+        <v/>
+      </c>
+      <c r="N16" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$16:$BD$16))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$16:$BD$16=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$16:$BD$16)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="5" t="n"/>
+      <c r="C17" s="5" t="n"/>
+      <c r="D17" s="5" t="n"/>
+      <c r="E17" s="5" t="n"/>
+      <c r="F17" s="5" t="n"/>
+      <c r="G17" s="5" t="n"/>
+      <c r="I17" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$17:$BD$17))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$17:$BD$17=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$17:$BD$17)))</f>
+        <v/>
+      </c>
+      <c r="J17" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$17:$BD$17))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$17:$BD$17=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$17:$BD$17)))</f>
+        <v/>
+      </c>
+      <c r="K17" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$17:$BD$17))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$17:$BD$17=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$17:$BD$17)))</f>
+        <v/>
+      </c>
+      <c r="L17" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$17:$BD$17))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$17:$BD$17=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$17:$BD$17)))</f>
+        <v/>
+      </c>
+      <c r="M17" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$17:$BD$17))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$17:$BD$17=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$17:$BD$17)))</f>
+        <v/>
+      </c>
+      <c r="N17" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$17:$BD$17))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$17:$BD$17=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$17:$BD$17)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="5" t="n"/>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="5" t="n"/>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="5" t="n"/>
+      <c r="G18" s="5" t="n"/>
+      <c r="I18" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$18:$BD$18))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$18:$BD$18=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$18:$BD$18)))</f>
+        <v/>
+      </c>
+      <c r="J18" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$18:$BD$18))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$18:$BD$18=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$18:$BD$18)))</f>
+        <v/>
+      </c>
+      <c r="K18" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$18:$BD$18))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$18:$BD$18=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$18:$BD$18)))</f>
+        <v/>
+      </c>
+      <c r="L18" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$18:$BD$18))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$18:$BD$18=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$18:$BD$18)))</f>
+        <v/>
+      </c>
+      <c r="M18" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$18:$BD$18))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$18:$BD$18=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$18:$BD$18)))</f>
+        <v/>
+      </c>
+      <c r="N18" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$18:$BD$18))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$18:$BD$18=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$18:$BD$18)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="5" t="n"/>
+      <c r="C19" s="5" t="n"/>
+      <c r="D19" s="5" t="n"/>
+      <c r="E19" s="5" t="n"/>
+      <c r="F19" s="5" t="n"/>
+      <c r="G19" s="5" t="n"/>
+      <c r="I19" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$19:$BD$19))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$19:$BD$19=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$19:$BD$19)))</f>
+        <v/>
+      </c>
+      <c r="J19" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$19:$BD$19))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$19:$BD$19=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$19:$BD$19)))</f>
+        <v/>
+      </c>
+      <c r="K19" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$19:$BD$19))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$19:$BD$19=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$19:$BD$19)))</f>
+        <v/>
+      </c>
+      <c r="L19" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$19:$BD$19))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$19:$BD$19=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$19:$BD$19)))</f>
+        <v/>
+      </c>
+      <c r="M19" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$19:$BD$19))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$19:$BD$19=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$19:$BD$19)))</f>
+        <v/>
+      </c>
+      <c r="N19" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$19:$BD$19))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$19:$BD$19=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$19:$BD$19)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="5" t="n"/>
+      <c r="C20" s="5" t="n"/>
+      <c r="D20" s="5" t="n"/>
+      <c r="E20" s="5" t="n"/>
+      <c r="F20" s="5" t="n"/>
+      <c r="G20" s="5" t="n"/>
+      <c r="I20" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$20:$BD$20))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$20:$BD$20=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$20:$BD$20)))</f>
+        <v/>
+      </c>
+      <c r="J20" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$20:$BD$20))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$20:$BD$20=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$20:$BD$20)))</f>
+        <v/>
+      </c>
+      <c r="K20" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$20:$BD$20))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$20:$BD$20=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$20:$BD$20)))</f>
+        <v/>
+      </c>
+      <c r="L20" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$20:$BD$20))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$20:$BD$20=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$20:$BD$20)))</f>
+        <v/>
+      </c>
+      <c r="M20" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$20:$BD$20))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$20:$BD$20=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$20:$BD$20)))</f>
+        <v/>
+      </c>
+      <c r="N20" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$20:$BD$20))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$20:$BD$20=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$20:$BD$20)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="5" t="n"/>
+      <c r="C21" s="5" t="n"/>
+      <c r="D21" s="5" t="n"/>
+      <c r="E21" s="5" t="n"/>
+      <c r="F21" s="5" t="n"/>
+      <c r="G21" s="5" t="n"/>
+      <c r="I21" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$21:$BD$21))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$21:$BD$21=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$21:$BD$21)))</f>
+        <v/>
+      </c>
+      <c r="J21" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$21:$BD$21))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$21:$BD$21=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$21:$BD$21)))</f>
+        <v/>
+      </c>
+      <c r="K21" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$21:$BD$21))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$21:$BD$21=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$21:$BD$21)))</f>
+        <v/>
+      </c>
+      <c r="L21" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$21:$BD$21))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$21:$BD$21=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$21:$BD$21)))</f>
+        <v/>
+      </c>
+      <c r="M21" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$21:$BD$21))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$21:$BD$21=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$21:$BD$21)))</f>
+        <v/>
+      </c>
+      <c r="N21" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$21:$BD$21))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$21:$BD$21=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$21:$BD$21)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="n"/>
+      <c r="I22" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$22:$BD$22))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$22:$BD$22=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$22:$BD$22)))</f>
+        <v/>
+      </c>
+      <c r="J22" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$22:$BD$22))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$22:$BD$22=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$22:$BD$22)))</f>
+        <v/>
+      </c>
+      <c r="K22" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$22:$BD$22))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$22:$BD$22=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$22:$BD$22)))</f>
+        <v/>
+      </c>
+      <c r="L22" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$22:$BD$22))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$22:$BD$22=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$22:$BD$22)))</f>
+        <v/>
+      </c>
+      <c r="M22" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$22:$BD$22))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$22:$BD$22=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$22:$BD$22)))</f>
+        <v/>
+      </c>
+      <c r="N22" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$22:$BD$22))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$22:$BD$22=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$22:$BD$22)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="5" t="n"/>
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="5" t="n"/>
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="5" t="n"/>
+      <c r="G23" s="5" t="n"/>
+      <c r="I23" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$23:$BD$23))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$23:$BD$23=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$23:$BD$23)))</f>
+        <v/>
+      </c>
+      <c r="J23" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$23:$BD$23))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$23:$BD$23=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$23:$BD$23)))</f>
+        <v/>
+      </c>
+      <c r="K23" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$23:$BD$23))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$23:$BD$23=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$23:$BD$23)))</f>
+        <v/>
+      </c>
+      <c r="L23" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$23:$BD$23))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$23:$BD$23=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$23:$BD$23)))</f>
+        <v/>
+      </c>
+      <c r="M23" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$23:$BD$23))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$23:$BD$23=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$23:$BD$23)))</f>
+        <v/>
+      </c>
+      <c r="N23" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$23:$BD$23))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$23:$BD$23=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$23:$BD$23)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="5" t="n"/>
+      <c r="C24" s="5" t="n"/>
+      <c r="D24" s="5" t="n"/>
+      <c r="E24" s="5" t="n"/>
+      <c r="F24" s="5" t="n"/>
+      <c r="G24" s="5" t="n"/>
+      <c r="I24" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$24:$BD$24))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$24:$BD$24=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$24:$BD$24)))</f>
+        <v/>
+      </c>
+      <c r="J24" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$24:$BD$24))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$24:$BD$24=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$24:$BD$24)))</f>
+        <v/>
+      </c>
+      <c r="K24" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$24:$BD$24))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$24:$BD$24=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$24:$BD$24)))</f>
+        <v/>
+      </c>
+      <c r="L24" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$24:$BD$24))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$24:$BD$24=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$24:$BD$24)))</f>
+        <v/>
+      </c>
+      <c r="M24" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$24:$BD$24))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$24:$BD$24=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$24:$BD$24)))</f>
+        <v/>
+      </c>
+      <c r="N24" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$24:$BD$24))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$24:$BD$24=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$24:$BD$24)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="5" t="n"/>
+      <c r="C25" s="5" t="n"/>
+      <c r="D25" s="5" t="n"/>
+      <c r="E25" s="5" t="n"/>
+      <c r="F25" s="5" t="n"/>
+      <c r="G25" s="5" t="n"/>
+      <c r="I25" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$25:$BD$25))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$25:$BD$25=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$25:$BD$25)))</f>
+        <v/>
+      </c>
+      <c r="J25" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$25:$BD$25))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$25:$BD$25=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$25:$BD$25)))</f>
+        <v/>
+      </c>
+      <c r="K25" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$25:$BD$25))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$25:$BD$25=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$25:$BD$25)))</f>
+        <v/>
+      </c>
+      <c r="L25" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$25:$BD$25))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$25:$BD$25=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$25:$BD$25)))</f>
+        <v/>
+      </c>
+      <c r="M25" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$25:$BD$25))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$25:$BD$25=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$25:$BD$25)))</f>
+        <v/>
+      </c>
+      <c r="N25" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$25:$BD$25))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$25:$BD$25=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$25:$BD$25)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="5" t="n"/>
+      <c r="C26" s="5" t="n"/>
+      <c r="D26" s="5" t="n"/>
+      <c r="E26" s="5" t="n"/>
+      <c r="F26" s="5" t="n"/>
+      <c r="G26" s="5" t="n"/>
+      <c r="I26" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$26:$BD$26))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$26:$BD$26=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$26:$BD$26)))</f>
+        <v/>
+      </c>
+      <c r="J26" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$26:$BD$26))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$26:$BD$26=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$26:$BD$26)))</f>
+        <v/>
+      </c>
+      <c r="K26" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$26:$BD$26))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$26:$BD$26=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$26:$BD$26)))</f>
+        <v/>
+      </c>
+      <c r="L26" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$26:$BD$26))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$26:$BD$26=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$26:$BD$26)))</f>
+        <v/>
+      </c>
+      <c r="M26" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$26:$BD$26))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$26:$BD$26=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$26:$BD$26)))</f>
+        <v/>
+      </c>
+      <c r="N26" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$26:$BD$26))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$26:$BD$26=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$26:$BD$26)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="5" t="n"/>
+      <c r="C27" s="5" t="n"/>
+      <c r="D27" s="5" t="n"/>
+      <c r="E27" s="5" t="n"/>
+      <c r="F27" s="5" t="n"/>
+      <c r="G27" s="5" t="n"/>
+      <c r="I27" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$27:$BD$27))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$27:$BD$27=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$27:$BD$27)))</f>
+        <v/>
+      </c>
+      <c r="J27" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$27:$BD$27))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$27:$BD$27=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$27:$BD$27)))</f>
+        <v/>
+      </c>
+      <c r="K27" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$27:$BD$27))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$27:$BD$27=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$27:$BD$27)))</f>
+        <v/>
+      </c>
+      <c r="L27" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$27:$BD$27))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$27:$BD$27=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$27:$BD$27)))</f>
+        <v/>
+      </c>
+      <c r="M27" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$27:$BD$27))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$27:$BD$27=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$27:$BD$27)))</f>
+        <v/>
+      </c>
+      <c r="N27" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$27:$BD$27))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$27:$BD$27=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$27:$BD$27)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="5" t="n"/>
+      <c r="C28" s="5" t="n"/>
+      <c r="D28" s="5" t="n"/>
+      <c r="E28" s="5" t="n"/>
+      <c r="F28" s="5" t="n"/>
+      <c r="G28" s="5" t="n"/>
+      <c r="I28" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$28:$BD$28))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$28:$BD$28=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$28:$BD$28)))</f>
+        <v/>
+      </c>
+      <c r="J28" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$28:$BD$28))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$28:$BD$28=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$28:$BD$28)))</f>
+        <v/>
+      </c>
+      <c r="K28" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$28:$BD$28))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$28:$BD$28=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$28:$BD$28)))</f>
+        <v/>
+      </c>
+      <c r="L28" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$28:$BD$28))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$28:$BD$28=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$28:$BD$28)))</f>
+        <v/>
+      </c>
+      <c r="M28" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$28:$BD$28))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$28:$BD$28=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$28:$BD$28)))</f>
+        <v/>
+      </c>
+      <c r="N28" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$28:$BD$28))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$28:$BD$28=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$28:$BD$28)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="5" t="n"/>
+      <c r="C29" s="5" t="n"/>
+      <c r="D29" s="5" t="n"/>
+      <c r="E29" s="5" t="n"/>
+      <c r="F29" s="5" t="n"/>
+      <c r="G29" s="5" t="n"/>
+      <c r="I29" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$29:$BD$29))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$29:$BD$29=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$29:$BD$29)))</f>
+        <v/>
+      </c>
+      <c r="J29" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$29:$BD$29))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$29:$BD$29=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$29:$BD$29)))</f>
+        <v/>
+      </c>
+      <c r="K29" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$29:$BD$29))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$29:$BD$29=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$29:$BD$29)))</f>
+        <v/>
+      </c>
+      <c r="L29" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$29:$BD$29))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$29:$BD$29=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$29:$BD$29)))</f>
+        <v/>
+      </c>
+      <c r="M29" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$29:$BD$29))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$29:$BD$29=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$29:$BD$29)))</f>
+        <v/>
+      </c>
+      <c r="N29" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$29:$BD$29))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$29:$BD$29=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$29:$BD$29)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="5" t="n"/>
+      <c r="C30" s="5" t="n"/>
+      <c r="D30" s="5" t="n"/>
+      <c r="E30" s="5" t="n"/>
+      <c r="F30" s="5" t="n"/>
+      <c r="G30" s="5" t="n"/>
+      <c r="I30" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$30:$BD$30))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$30:$BD$30=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$30:$BD$30)))</f>
+        <v/>
+      </c>
+      <c r="J30" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$30:$BD$30))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$30:$BD$30=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$30:$BD$30)))</f>
+        <v/>
+      </c>
+      <c r="K30" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$30:$BD$30))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$30:$BD$30=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$30:$BD$30)))</f>
+        <v/>
+      </c>
+      <c r="L30" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$30:$BD$30))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$30:$BD$30=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$30:$BD$30)))</f>
+        <v/>
+      </c>
+      <c r="M30" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$30:$BD$30))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$30:$BD$30=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$30:$BD$30)))</f>
+        <v/>
+      </c>
+      <c r="N30" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$30:$BD$30))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$30:$BD$30=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$30:$BD$30)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="I31" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$31:$BD$31))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$31:$BD$31=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$31:$BD$31)))</f>
+        <v/>
+      </c>
+      <c r="J31" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$31:$BD$31))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$31:$BD$31=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$31:$BD$31)))</f>
+        <v/>
+      </c>
+      <c r="K31" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$31:$BD$31))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$31:$BD$31=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$31:$BD$31)))</f>
+        <v/>
+      </c>
+      <c r="L31" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$31:$BD$31))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$31:$BD$31=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$31:$BD$31)))</f>
+        <v/>
+      </c>
+      <c r="M31" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$31:$BD$31))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$31:$BD$31=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$31:$BD$31)))</f>
+        <v/>
+      </c>
+      <c r="N31" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$31:$BD$31))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$31:$BD$31=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$31:$BD$31)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="5" t="n"/>
+      <c r="C32" s="5" t="n"/>
+      <c r="D32" s="5" t="n"/>
+      <c r="E32" s="5" t="n"/>
+      <c r="F32" s="5" t="n"/>
+      <c r="G32" s="5" t="n"/>
+      <c r="I32" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$32:$BD$32))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$32:$BD$32=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$32:$BD$32)))</f>
+        <v/>
+      </c>
+      <c r="J32" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$32:$BD$32))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$32:$BD$32=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$32:$BD$32)))</f>
+        <v/>
+      </c>
+      <c r="K32" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$32:$BD$32))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$32:$BD$32=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$32:$BD$32)))</f>
+        <v/>
+      </c>
+      <c r="L32" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$32:$BD$32))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$32:$BD$32=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$32:$BD$32)))</f>
+        <v/>
+      </c>
+      <c r="M32" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$32:$BD$32))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$32:$BD$32=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$32:$BD$32)))</f>
+        <v/>
+      </c>
+      <c r="N32" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$32:$BD$32))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$32:$BD$32=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$32:$BD$32)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="5" t="n"/>
+      <c r="C33" s="5" t="n"/>
+      <c r="D33" s="5" t="n"/>
+      <c r="E33" s="5" t="n"/>
+      <c r="F33" s="5" t="n"/>
+      <c r="G33" s="5" t="n"/>
+      <c r="I33" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$33:$BD$33))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$33:$BD$33=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$33:$BD$33)))</f>
+        <v/>
+      </c>
+      <c r="J33" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$33:$BD$33))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$33:$BD$33=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$33:$BD$33)))</f>
+        <v/>
+      </c>
+      <c r="K33" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$33:$BD$33))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$33:$BD$33=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$33:$BD$33)))</f>
+        <v/>
+      </c>
+      <c r="L33" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$33:$BD$33))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$33:$BD$33=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$33:$BD$33)))</f>
+        <v/>
+      </c>
+      <c r="M33" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$33:$BD$33))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$33:$BD$33=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$33:$BD$33)))</f>
+        <v/>
+      </c>
+      <c r="N33" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$33:$BD$33))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$33:$BD$33=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$33:$BD$33)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="5" t="n"/>
+      <c r="C34" s="5" t="n"/>
+      <c r="D34" s="5" t="n"/>
+      <c r="E34" s="5" t="n"/>
+      <c r="F34" s="5" t="n"/>
+      <c r="G34" s="5" t="n"/>
+      <c r="I34" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$34:$BD$34))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$34:$BD$34=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$34:$BD$34)))</f>
+        <v/>
+      </c>
+      <c r="J34" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$34:$BD$34))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$34:$BD$34=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$34:$BD$34)))</f>
+        <v/>
+      </c>
+      <c r="K34" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$34:$BD$34))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$34:$BD$34=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$34:$BD$34)))</f>
+        <v/>
+      </c>
+      <c r="L34" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$34:$BD$34))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$34:$BD$34=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$34:$BD$34)))</f>
+        <v/>
+      </c>
+      <c r="M34" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$34:$BD$34))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$34:$BD$34=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$34:$BD$34)))</f>
+        <v/>
+      </c>
+      <c r="N34" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$34:$BD$34))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$34:$BD$34=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$34:$BD$34)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="5" t="n"/>
+      <c r="C35" s="5" t="n"/>
+      <c r="D35" s="5" t="n"/>
+      <c r="E35" s="5" t="n"/>
+      <c r="F35" s="5" t="n"/>
+      <c r="G35" s="5" t="n"/>
+      <c r="I35" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$35:$BD$35))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$35:$BD$35=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$35:$BD$35)))</f>
+        <v/>
+      </c>
+      <c r="J35" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$35:$BD$35))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$35:$BD$35=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$35:$BD$35)))</f>
+        <v/>
+      </c>
+      <c r="K35" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$35:$BD$35))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$35:$BD$35=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$35:$BD$35)))</f>
+        <v/>
+      </c>
+      <c r="L35" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$35:$BD$35))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$35:$BD$35=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$35:$BD$35)))</f>
+        <v/>
+      </c>
+      <c r="M35" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$35:$BD$35))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$35:$BD$35=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$35:$BD$35)))</f>
+        <v/>
+      </c>
+      <c r="N35" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$35:$BD$35))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$35:$BD$35=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$35:$BD$35)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="5" t="n"/>
+      <c r="C36" s="5" t="n"/>
+      <c r="D36" s="5" t="n"/>
+      <c r="E36" s="5" t="n"/>
+      <c r="F36" s="5" t="n"/>
+      <c r="G36" s="5" t="n"/>
+      <c r="I36" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$36:$BD$36))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$36:$BD$36=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$36:$BD$36)))</f>
+        <v/>
+      </c>
+      <c r="J36" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$36:$BD$36))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$36:$BD$36=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$36:$BD$36)))</f>
+        <v/>
+      </c>
+      <c r="K36" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$36:$BD$36))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$36:$BD$36=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$36:$BD$36)))</f>
+        <v/>
+      </c>
+      <c r="L36" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$36:$BD$36))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$36:$BD$36=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$36:$BD$36)))</f>
+        <v/>
+      </c>
+      <c r="M36" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$36:$BD$36))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$36:$BD$36=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$36:$BD$36)))</f>
+        <v/>
+      </c>
+      <c r="N36" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$36:$BD$36))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$36:$BD$36=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$36:$BD$36)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="5" t="n"/>
+      <c r="C37" s="5" t="n"/>
+      <c r="D37" s="5" t="n"/>
+      <c r="E37" s="5" t="n"/>
+      <c r="F37" s="5" t="n"/>
+      <c r="G37" s="5" t="n"/>
+      <c r="I37" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$37:$BD$37))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$37:$BD$37=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$37:$BD$37)))</f>
+        <v/>
+      </c>
+      <c r="J37" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$37:$BD$37))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$37:$BD$37=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$37:$BD$37)))</f>
+        <v/>
+      </c>
+      <c r="K37" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$37:$BD$37))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$37:$BD$37=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$37:$BD$37)))</f>
+        <v/>
+      </c>
+      <c r="L37" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$37:$BD$37))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$37:$BD$37=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$37:$BD$37)))</f>
+        <v/>
+      </c>
+      <c r="M37" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$37:$BD$37))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$37:$BD$37=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$37:$BD$37)))</f>
+        <v/>
+      </c>
+      <c r="N37" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$37:$BD$37))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$37:$BD$37=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$37:$BD$37)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="5" t="n"/>
+      <c r="C38" s="5" t="n"/>
+      <c r="D38" s="5" t="n"/>
+      <c r="E38" s="5" t="n"/>
+      <c r="F38" s="5" t="n"/>
+      <c r="G38" s="5" t="n"/>
+      <c r="I38" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$38:$BD$38))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$38:$BD$38=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$38:$BD$38)))</f>
+        <v/>
+      </c>
+      <c r="J38" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$38:$BD$38))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$38:$BD$38=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$38:$BD$38)))</f>
+        <v/>
+      </c>
+      <c r="K38" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$38:$BD$38))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$38:$BD$38=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$38:$BD$38)))</f>
+        <v/>
+      </c>
+      <c r="L38" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$38:$BD$38))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$38:$BD$38=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$38:$BD$38)))</f>
+        <v/>
+      </c>
+      <c r="M38" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$38:$BD$38))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$38:$BD$38=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$38:$BD$38)))</f>
+        <v/>
+      </c>
+      <c r="N38" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$38:$BD$38))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$38:$BD$38=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$38:$BD$38)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="5" t="n"/>
+      <c r="C39" s="5" t="n"/>
+      <c r="D39" s="5" t="n"/>
+      <c r="E39" s="5" t="n"/>
+      <c r="F39" s="5" t="n"/>
+      <c r="G39" s="5" t="n"/>
+      <c r="I39" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$39:$BD$39))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*(Marks!$B$39:$BD$39=1))/SUMPRODUCT((Marks!$B$2:$BD$2=I$3)*ISNUMBER(Marks!$B$39:$BD$39)))</f>
+        <v/>
+      </c>
+      <c r="J39" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$39:$BD$39))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*(Marks!$B$39:$BD$39=1))/SUMPRODUCT((Marks!$B$2:$BD$2=J$3)*ISNUMBER(Marks!$B$39:$BD$39)))</f>
+        <v/>
+      </c>
+      <c r="K39" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$39:$BD$39))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*(Marks!$B$39:$BD$39=1))/SUMPRODUCT((Marks!$B$2:$BD$2=K$3)*ISNUMBER(Marks!$B$39:$BD$39)))</f>
+        <v/>
+      </c>
+      <c r="L39" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$39:$BD$39))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*(Marks!$B$39:$BD$39=1))/SUMPRODUCT((Marks!$B$2:$BD$2=L$3)*ISNUMBER(Marks!$B$39:$BD$39)))</f>
+        <v/>
+      </c>
+      <c r="M39" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$39:$BD$39))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*(Marks!$B$39:$BD$39=1))/SUMPRODUCT((Marks!$B$2:$BD$2=M$3)*ISNUMBER(Marks!$B$39:$BD$39)))</f>
+        <v/>
+      </c>
+      <c r="N39" s="6">
+        <f>IF(SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$39:$BD$39))=0,"",SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*(Marks!$B$39:$BD$39=1))/SUMPRODUCT((Marks!$B$2:$BD$2=N$3)*ISNUMBER(Marks!$B$39:$BD$39)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>The room</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>Mean rating</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>Right rate</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>Rated 3 or 4, under half right</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Part 1. The week's rules, cold</t>
+        </is>
+      </c>
+      <c r="B43" s="7">
+        <f>IF(COUNT(B5:B39)=0,"",AVERAGE(B5:B39))</f>
+        <v/>
+      </c>
+      <c r="C43" s="6">
+        <f>IFERROR(INDEX(Tags!$D$5:$D$13,MATCH(1,Tags!$A$5:$A$13,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D43">
+        <f>SUMPRODUCT((B5:B39&gt;=3)*ISNUMBER(I5:I39)*(I5:I39&lt;0.5))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Part 2. Asking the warehouse</t>
+        </is>
+      </c>
+      <c r="B44" s="7">
+        <f>IF(COUNT(C5:C39)=0,"",AVERAGE(C5:C39))</f>
+        <v/>
+      </c>
+      <c r="C44" s="6">
+        <f>IFERROR(INDEX(Tags!$D$5:$D$13,MATCH(2,Tags!$A$5:$A$13,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D44">
+        <f>SUMPRODUCT((C5:C39&gt;=3)*ISNUMBER(J5:J39)*(J5:J39&lt;0.5))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Part 3. Joins that keep their rows</t>
+        </is>
+      </c>
+      <c r="B45" s="7">
+        <f>IF(COUNT(D5:D39)=0,"",AVERAGE(D5:D39))</f>
+        <v/>
+      </c>
+      <c r="C45" s="6">
+        <f>IFERROR(INDEX(Tags!$D$5:$D$13,MATCH(3,Tags!$A$5:$A$13,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D45">
+        <f>SUMPRODUCT((D5:D39&gt;=3)*ISNUMBER(K5:K39)*(K5:K39&lt;0.5))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Part 4. Windows: rank, lag and running totals</t>
+        </is>
+      </c>
+      <c r="B46" s="7">
+        <f>IF(COUNT(E5:E39)=0,"",AVERAGE(E5:E39))</f>
+        <v/>
+      </c>
+      <c r="C46" s="6">
+        <f>IFERROR(INDEX(Tags!$D$5:$D$13,MATCH(4,Tags!$A$5:$A$13,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D46">
+        <f>SUMPRODUCT((E5:E39&gt;=3)*ISNUMBER(L5:L39)*(L5:L39&lt;0.5))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Part 5. pandas and the last mile to Excel</t>
+        </is>
+      </c>
+      <c r="B47" s="7">
+        <f>IF(COUNT(F5:F39)=0,"",AVERAGE(F5:F39))</f>
+        <v/>
+      </c>
+      <c r="C47" s="6">
+        <f>IFERROR(INDEX(Tags!$D$5:$D$13,MATCH(5,Tags!$A$5:$A$13,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D47">
+        <f>SUMPRODUCT((F5:F39&gt;=3)*ISNUMBER(M5:M39)*(M5:M39&lt;0.5))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Part 6. Read the code, read the data</t>
+        </is>
+      </c>
+      <c r="B48" s="7">
+        <f>IF(COUNT(G5:G39)=0,"",AVERAGE(G5:G39))</f>
+        <v/>
+      </c>
+      <c r="C48" s="6">
+        <f>IFERROR(INDEX(Tags!$D$5:$D$13,MATCH(6,Tags!$A$5:$A$13,0)),"")</f>
+        <v/>
+      </c>
+      <c r="D48">
+        <f>SUMPRODUCT((G5:G39&gt;=3)*ISNUMBER(N5:N39)*(N5:N39&lt;0.5))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Week 2 Saturday v3: the paper raised after the blind sitting
Ten items rebuilt as several steps on an exhibit (Q8, Q10, Q11, Q15, Q16,
Q20, Q27, Q28, Q29, Q32), Q1 turned into worked arithmetic, Q5 and Q13
relabelled medium and Q34 hard, so 21 of 35 items are hard in fact. Every
give-away, cross-item leak and arguable key the sitting found is closed, the
public-case facts are corrected against their sources, the invented Part 6
company is no longer named, and every key is proved again.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01P7zaoR4dQ5pzBFnsX549JQ
</commit_message>
<xml_diff>
--- a/content/W02/SAT/answer-key/C2_W02_SAT_item_analysis_TRAINER.xlsx
+++ b/content/W02/SAT/answer-key/C2_W02_SAT_item_analysis_TRAINER.xlsx
@@ -2935,7 +2935,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>One correct option</t>
+          <t>Applied maths</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -2950,7 +2950,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>It prints 2 and 1. The true figures are 2.36 and 1.84, a fall of about 22 percent.</t>
         </is>
       </c>
       <c r="G5">
@@ -3180,7 +3180,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -3190,7 +3190,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>b</t>
         </is>
       </c>
       <c r="G9">
@@ -3370,7 +3370,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>c, e, a, d, b</t>
+          <t>e, f, b, c, a</t>
         </is>
       </c>
       <c r="G12">
@@ -3660,7 +3660,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -3670,7 +3670,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>c</t>
         </is>
       </c>
       <c r="G17">
@@ -4090,7 +4090,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>d</t>
         </is>
       </c>
       <c r="G24">
@@ -4495,7 +4495,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>One correct option</t>
+          <t>Applied maths</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -4510,7 +4510,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>B8 returns -0.5; the six rows average 1.0; the formula understates growth by 1.5 points and turns growth into a fall.</t>
         </is>
       </c>
       <c r="G31">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>b</t>
         </is>
       </c>
       <c r="G32">
@@ -4620,7 +4620,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -4630,7 +4630,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>0.60 dollars a trip</t>
+          <t>2.00 dollars, about 8.5 percent of the 23.50 dollars charged</t>
         </is>
       </c>
       <c r="G33">
@@ -4810,7 +4810,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>a</t>
         </is>
       </c>
       <c r="G36">
@@ -4920,7 +4920,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">

</xml_diff>

<commit_message>
W02 Saturday: the review's fixes to items and parts, rebuilt with the key proofs
Q32's stem routes every call whose total is over 1,000, so the first call
routed has one reading. Q12's options a and d both say 51, so the count no
longer finds the key. Q28's MergeError option no longer says the labels
repeat. Part 4 and Part 5 are renamed by the question each asks, Part 5's
opening names its three public cases as numbers people relied on and
Friday's protect list, and Part 6 opens on a drawing of who acts on which
table. Set 1 states that every paid order was paid in full and Q10 that
no order was paid short, which the proofs check on the warehouse. The
key's reasons lose their run tails and cite Friday for JPMorgan; Q14's
option d divides by the average, so no key is a lone length outlier.
No key moved; the proofs pass 33 of 33.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q6BoMrCz4psj5e3WRTrZh9
</commit_message>
<xml_diff>
--- a/content/W02/SAT/answer-key/C2_W02_SAT_item_analysis_TRAINER.xlsx
+++ b/content/W02/SAT/answer-key/C2_W02_SAT_item_analysis_TRAINER.xlsx
@@ -5863,7 +5863,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Part 4. Can the growth team act on Monday's table of 340 customers without checking it first?</t>
+          <t>Part 4. What must Monday's customer table check before the growth team acts on it?</t>
         </is>
       </c>
       <c r="C11">
@@ -5881,7 +5881,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Part 5. Which spreadsheet numbers can a director trust, in Monday's workbook and in three public cases?</t>
+          <t>Part 5. Which numbers in Monday's workbook can a director trust, and where did three public cases go wrong?</t>
         </is>
       </c>
       <c r="C12">
@@ -7999,7 +7999,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Part 4. Can the growth team act on Monday's table of 340 customers without checking it first?</t>
+          <t>Part 4. What must Monday's customer table check before the growth team acts on it?</t>
         </is>
       </c>
       <c r="B46" s="7">
@@ -8018,7 +8018,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Part 5. Which spreadsheet numbers can a director trust, in Monday's workbook and in three public cases?</t>
+          <t>Part 5. Which numbers in Monday's workbook can a director trust, and where did three public cases go wrong?</t>
         </is>
       </c>
       <c r="B47" s="7">

</xml_diff>